<commit_message>
Add shared to-do page, update churn project case study, and refresh progress/nav
- New todo.html + js/todo.js + css/todo.css + data/tasks.json: shared task tracker with activity history, documented in TASKS.md
- Add "To-do" nav link across index, job-tracker, progress, and projects pages
- index.html: replace churn placeholder card with real Subscriber Churn Early-Warning & LTV Segmentation case study and results
- progress.html: rewrite intro copy and section labels, link out to the new to-do list
- Update data/progress-data.js, data/projects.json, job-applications.xlsx, and project card image

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\EileenIp.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE4688D3-E2B7-4456-8ED6-AC4328B079A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1ACFC3EB-A08A-483A-960A-CC88FEF3545A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1820" yWindow="1820" windowWidth="14400" windowHeight="8710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Applications" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Applications!$A$1:$AC$94</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="359">
   <si>
     <t>Company</t>
   </si>
@@ -1059,6 +1060,63 @@
   </si>
   <si>
     <t>Finished Assessment</t>
+  </si>
+  <si>
+    <t>business data analyst project intern (GBS)</t>
+  </si>
+  <si>
+    <t>2000-5000 per month</t>
+  </si>
+  <si>
+    <t>Sports Consultancy and data analyst intern</t>
+  </si>
+  <si>
+    <t>Futures Sport &amp; entertainment</t>
+  </si>
+  <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>Didi</t>
+  </si>
+  <si>
+    <t>operations intern</t>
+  </si>
+  <si>
+    <t>Game Reaserch Development intern, engine reasearch</t>
+  </si>
+  <si>
+    <t>tencent</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>information systems and technology</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>student training and totation program intern</t>
+  </si>
+  <si>
+    <t>2 years</t>
+  </si>
+  <si>
+    <t>bytedance</t>
+  </si>
+  <si>
+    <t>ai sales intern</t>
+  </si>
+  <si>
+    <t>binance</t>
+  </si>
+  <si>
+    <t>BAP data analyst</t>
+  </si>
+  <si>
+    <t>3 month</t>
   </si>
 </sst>
 </file>
@@ -2064,7 +2122,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC98"/>
+  <dimension ref="A1:AC106"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -6917,7 +6975,7 @@
         <v>33</v>
       </c>
       <c r="M95" s="25" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="P95" s="6" t="s">
         <v>327</v>
@@ -7026,6 +7084,142 @@
       </c>
       <c r="U98" s="7" t="s">
         <v>320</v>
+      </c>
+    </row>
+    <row r="99" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A99" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="B99" t="s">
+        <v>340</v>
+      </c>
+      <c r="C99" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D99" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F99" s="6">
+        <v>46387</v>
+      </c>
+      <c r="H99" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="M99" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="T99" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="100" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A100" s="25" t="s">
+        <v>343</v>
+      </c>
+      <c r="B100" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="C100" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D100" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H100" s="25" t="s">
+        <v>344</v>
+      </c>
+      <c r="M100" s="25" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="101" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A101" s="25" t="s">
+        <v>345</v>
+      </c>
+      <c r="B101" s="25" t="s">
+        <v>346</v>
+      </c>
+      <c r="C101" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D101" s="25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="102" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A102" s="25" t="s">
+        <v>348</v>
+      </c>
+      <c r="B102" t="s">
+        <v>347</v>
+      </c>
+      <c r="C102" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D102" s="25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="103" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A103" s="25" t="s">
+        <v>349</v>
+      </c>
+      <c r="B103" t="s">
+        <v>350</v>
+      </c>
+      <c r="C103" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D103" s="25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="104" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A104" s="25" t="s">
+        <v>351</v>
+      </c>
+      <c r="B104" t="s">
+        <v>352</v>
+      </c>
+      <c r="C104" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D104" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="R104" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="105" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A105" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="B105" t="s">
+        <v>355</v>
+      </c>
+      <c r="C105" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D105" s="25" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="106" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A106" s="25" t="s">
+        <v>356</v>
+      </c>
+      <c r="B106" t="s">
+        <v>357</v>
+      </c>
+      <c r="C106" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="D106" s="25" t="s">
+        <v>279</v>
+      </c>
+      <c r="R106" t="s">
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -7127,7 +7321,7 @@
     <dataValidation type="list" allowBlank="1" sqref="D86:D495" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"NSW,VIC,QLD,WA,SA,TAS,ACT,NT,Remote,Hybrid,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H96:H495" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H96:H98 H100:H495" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Seek,LinkedIn,Company Website,University Portal,Indeed,Referral,Career Fair,Other"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="K86:K495" xr:uid="{00000000-0002-0000-0000-000003000000}">

</xml_diff>

<commit_message>
job-tracker: update application statuses and log new applications
New: Apple, Didi, SAP, Tencent, TikTok. Status updates: two withdrawn,
several rejected, a few moved to Applied. Removed two stale To Apply
rows (Canva, Woolworths) past their deadline.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -20,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="0&quot; days&quot;"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -196,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -256,6 +257,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1085,7 +1088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC106"/>
+  <dimension ref="A1:AC96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="31" min="1" max="1"/>
@@ -3449,12 +3452,12 @@
     <row r="32" ht="18" customHeight="1" s="31">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>canva</t>
+          <t>Allianz</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>data analytics</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -3469,7 +3472,7 @@
       </c>
       <c r="E32" s="13" t="n"/>
       <c r="F32" s="14" t="n">
-        <v>46157</v>
+        <v>46147</v>
       </c>
       <c r="G32" s="13" t="n"/>
       <c r="H32" s="13" t="inlineStr">
@@ -3483,30 +3486,20 @@
       <c r="L32" s="13" t="n"/>
       <c r="M32" s="13" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="N32" s="13" t="n"/>
       <c r="O32" s="13" t="n"/>
-      <c r="P32" s="14" t="n">
-        <v>46434</v>
-      </c>
+      <c r="P32" s="13" t="n"/>
       <c r="Q32" s="17" t="n"/>
       <c r="R32" s="18">
-        <f>IF(AND(P32&lt;&gt;"",Q32&lt;&gt;""),Q32-P32,"")</f>
+        <f>IF(AND(P34&lt;&gt;"",Q34&lt;&gt;""),Q34-P34,"")</f>
         <v/>
       </c>
       <c r="S32" s="13" t="n"/>
-      <c r="T32" s="13" t="inlineStr">
-        <is>
-          <t>95k - 119k</t>
-        </is>
-      </c>
-      <c r="U32" s="20" t="inlineStr">
-        <is>
-          <t>1-25</t>
-        </is>
-      </c>
+      <c r="T32" s="13" t="n"/>
+      <c r="U32" s="20" t="n"/>
       <c r="V32" s="13" t="n"/>
       <c r="W32" s="13" t="n"/>
       <c r="X32" s="13" t="n"/>
@@ -3519,23 +3512,31 @@
     <row r="33" ht="18" customHeight="1" s="31">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>tiktok</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="n"/>
+          <t>FMD</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Project Grace: Data Analyst</t>
+        </is>
+      </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n"/>
-      <c r="G33" s="13" t="n"/>
+          <t>VIC, NSW</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="n">
+        <v>46112</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>46108</v>
+      </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -3547,7 +3548,7 @@
       <c r="L33" s="13" t="n"/>
       <c r="M33" s="13" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="N33" s="13" t="n"/>
@@ -3555,30 +3556,46 @@
       <c r="P33" s="13" t="n"/>
       <c r="Q33" s="17" t="n"/>
       <c r="R33" s="18">
-        <f>IF(AND(P33&lt;&gt;"",Q33&lt;&gt;""),Q33-P33,"")</f>
+        <f>IF(AND(P35&lt;&gt;"",Q35&lt;&gt;""),Q35-P35,"")</f>
         <v/>
       </c>
       <c r="S33" s="13" t="n"/>
-      <c r="T33" s="13" t="n"/>
-      <c r="U33" s="20" t="n"/>
+      <c r="T33" s="13" t="inlineStr">
+        <is>
+          <t>67k-70k</t>
+        </is>
+      </c>
+      <c r="U33" s="20" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
       <c r="V33" s="13" t="n"/>
       <c r="W33" s="13" t="n"/>
       <c r="X33" s="13" t="n"/>
       <c r="Y33" s="13" t="n"/>
       <c r="Z33" s="13" t="n"/>
-      <c r="AA33" s="13" t="n"/>
-      <c r="AB33" s="13" t="n"/>
+      <c r="AA33" s="13" t="inlineStr">
+        <is>
+          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
+        </is>
+      </c>
+      <c r="AB33" s="13" t="inlineStr">
+        <is>
+          <t>Vendor Performance &amp; Procurement Analytics Dashboard, Credit Fraud Detection Classifier Analysis, Customer Segmentation in Bank Marketing Campaign Presentation, Customer Churn Forecasting Analysis in Telecom Services</t>
+        </is>
+      </c>
       <c r="AC33" s="13" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1" s="31">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Allianz</t>
+          <t>Qantas</t>
         </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>data analytics</t>
+          <t>data &amp; analytics</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -3586,16 +3603,18 @@
           <t>Graduate Program</t>
         </is>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
       <c r="E34" s="13" t="n"/>
       <c r="F34" s="14" t="n">
-        <v>46147</v>
-      </c>
-      <c r="G34" s="13" t="n"/>
+        <v>46166</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>46166</v>
+      </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -3615,7 +3634,7 @@
       <c r="P34" s="13" t="n"/>
       <c r="Q34" s="17" t="n"/>
       <c r="R34" s="18">
-        <f>IF(AND(P34&lt;&gt;"",Q34&lt;&gt;""),Q34-P34,"")</f>
+        <f>IF(AND(P36&lt;&gt;"",Q36&lt;&gt;""),Q36-P36,"")</f>
         <v/>
       </c>
       <c r="S34" s="13" t="n"/>
@@ -3626,19 +3645,27 @@
       <c r="X34" s="13" t="n"/>
       <c r="Y34" s="13" t="n"/>
       <c r="Z34" s="13" t="n"/>
-      <c r="AA34" s="13" t="n"/>
-      <c r="AB34" s="13" t="n"/>
+      <c r="AA34" s="13" t="inlineStr">
+        <is>
+          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
+        </is>
+      </c>
+      <c r="AB34" s="13" t="inlineStr">
+        <is>
+          <t>Hotel Customer Feedback Analytics Dashboard, Shopify Sales &amp; Customer Funnel Analytics Dashboard, Customer Churn Forecasting Analysis in Telecom Services, Customer Segmentation in Marketing Bank Campaigns Presentation</t>
+        </is>
+      </c>
       <c r="AC34" s="13" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1" s="31">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>FMD</t>
+          <t>RSM</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Project Grace: Data Analyst</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -3648,15 +3675,15 @@
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>VIC, NSW</t>
-        </is>
-      </c>
-      <c r="E35" s="14" t="n"/>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="n"/>
       <c r="F35" s="14" t="n">
-        <v>46112</v>
+        <v>46103</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>46108</v>
+        <v>46102</v>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
@@ -3674,21 +3701,23 @@
       </c>
       <c r="N35" s="13" t="n"/>
       <c r="O35" s="13" t="n"/>
-      <c r="P35" s="13" t="n"/>
+      <c r="P35" s="14" t="n">
+        <v>46419</v>
+      </c>
       <c r="Q35" s="17" t="n"/>
       <c r="R35" s="18">
-        <f>IF(AND(P35&lt;&gt;"",Q35&lt;&gt;""),Q35-P35,"")</f>
+        <f>IF(AND(P37&lt;&gt;"",Q37&lt;&gt;""),Q37-P37,"")</f>
         <v/>
       </c>
       <c r="S35" s="13" t="n"/>
       <c r="T35" s="13" t="inlineStr">
         <is>
-          <t>67k-70k</t>
+          <t>67-70k</t>
         </is>
       </c>
       <c r="U35" s="20" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="V35" s="13" t="n"/>
@@ -3703,7 +3732,7 @@
       </c>
       <c r="AB35" s="13" t="inlineStr">
         <is>
-          <t>Vendor Performance &amp; Procurement Analytics Dashboard, Credit Fraud Detection Classifier Analysis, Customer Segmentation in Bank Marketing Campaign Presentation, Customer Churn Forecasting Analysis in Telecom Services</t>
+          <t>Insurance Risk &amp; Claims Analysis Dashboard, Bank Loan Application Tracking Dashboard, Credit Fraud Detection Classifier</t>
         </is>
       </c>
       <c r="AC35" s="13" t="n"/>
@@ -3711,12 +3740,12 @@
     <row r="36" ht="18" customHeight="1" s="31">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>Qantas</t>
+          <t>amazon</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>data &amp; analytics</t>
+          <t>Graduate Brand Analyst,</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -3724,18 +3753,16 @@
           <t>Graduate Program</t>
         </is>
       </c>
-      <c r="D36" s="21" t="inlineStr">
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
       <c r="E36" s="13" t="n"/>
       <c r="F36" s="14" t="n">
-        <v>46166</v>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>46166</v>
-      </c>
+        <v>46147</v>
+      </c>
+      <c r="G36" s="13" t="n"/>
       <c r="H36" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -3745,17 +3772,15 @@
       <c r="J36" s="13" t="n"/>
       <c r="K36" s="13" t="n"/>
       <c r="L36" s="13" t="n"/>
-      <c r="M36" s="13" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
+      <c r="M36" s="13" t="n"/>
       <c r="N36" s="13" t="n"/>
       <c r="O36" s="13" t="n"/>
-      <c r="P36" s="13" t="n"/>
+      <c r="P36" s="14" t="n">
+        <v>46204</v>
+      </c>
       <c r="Q36" s="17" t="n"/>
       <c r="R36" s="18">
-        <f>IF(AND(P36&lt;&gt;"",Q36&lt;&gt;""),Q36-P36,"")</f>
+        <f>IF(AND(P38&lt;&gt;"",Q38&lt;&gt;""),Q38-P38,"")</f>
         <v/>
       </c>
       <c r="S36" s="13" t="n"/>
@@ -3766,29 +3791,17 @@
       <c r="X36" s="13" t="n"/>
       <c r="Y36" s="13" t="n"/>
       <c r="Z36" s="13" t="n"/>
-      <c r="AA36" s="13" t="inlineStr">
-        <is>
-          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
-        </is>
-      </c>
-      <c r="AB36" s="13" t="inlineStr">
-        <is>
-          <t>Hotel Customer Feedback Analytics Dashboard, Shopify Sales &amp; Customer Funnel Analytics Dashboard, Customer Churn Forecasting Analysis in Telecom Services, Customer Segmentation in Marketing Bank Campaigns Presentation</t>
-        </is>
-      </c>
+      <c r="AA36" s="13" t="n"/>
+      <c r="AB36" s="13" t="n"/>
       <c r="AC36" s="13" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="31">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>RSM</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Data Analytics</t>
-        </is>
-      </c>
+          <t>anz</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="n"/>
       <c r="C37" s="13" t="inlineStr">
         <is>
           <t>Graduate Program</t>
@@ -3796,16 +3809,12 @@
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E37" s="13" t="n"/>
-      <c r="F37" s="14" t="n">
-        <v>46103</v>
-      </c>
-      <c r="G37" s="14" t="n">
-        <v>46102</v>
-      </c>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="13" t="n"/>
       <c r="H37" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -3815,58 +3824,36 @@
       <c r="J37" s="13" t="n"/>
       <c r="K37" s="13" t="n"/>
       <c r="L37" s="13" t="n"/>
-      <c r="M37" s="13" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
+      <c r="M37" s="13" t="n"/>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>
-      <c r="P37" s="14" t="n">
-        <v>46419</v>
-      </c>
+      <c r="P37" s="13" t="n"/>
       <c r="Q37" s="17" t="n"/>
       <c r="R37" s="18">
-        <f>IF(AND(P37&lt;&gt;"",Q37&lt;&gt;""),Q37-P37,"")</f>
+        <f>IF(AND(P39&lt;&gt;"",Q39&lt;&gt;""),Q39-P39,"")</f>
         <v/>
       </c>
       <c r="S37" s="13" t="n"/>
-      <c r="T37" s="13" t="inlineStr">
-        <is>
-          <t>67-70k</t>
-        </is>
-      </c>
-      <c r="U37" s="20" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
+      <c r="T37" s="13" t="n"/>
+      <c r="U37" s="20" t="n"/>
       <c r="V37" s="13" t="n"/>
       <c r="W37" s="13" t="n"/>
       <c r="X37" s="13" t="n"/>
       <c r="Y37" s="13" t="n"/>
       <c r="Z37" s="13" t="n"/>
-      <c r="AA37" s="13" t="inlineStr">
-        <is>
-          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
-        </is>
-      </c>
-      <c r="AB37" s="13" t="inlineStr">
-        <is>
-          <t>Insurance Risk &amp; Claims Analysis Dashboard, Bank Loan Application Tracking Dashboard, Credit Fraud Detection Classifier</t>
-        </is>
-      </c>
+      <c r="AA37" s="13" t="n"/>
+      <c r="AB37" s="13" t="n"/>
       <c r="AC37" s="13" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1" s="31">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>bcg</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Graduate Brand Analyst,</t>
+          <t>consulting</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -3881,7 +3868,7 @@
       </c>
       <c r="E38" s="13" t="n"/>
       <c r="F38" s="14" t="n">
-        <v>46147</v>
+        <v>46085</v>
       </c>
       <c r="G38" s="13" t="n"/>
       <c r="H38" s="13" t="inlineStr">
@@ -3896,12 +3883,10 @@
       <c r="M38" s="13" t="n"/>
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="13" t="n"/>
-      <c r="P38" s="14" t="n">
-        <v>46204</v>
-      </c>
+      <c r="P38" s="13" t="n"/>
       <c r="Q38" s="17" t="n"/>
       <c r="R38" s="18">
-        <f>IF(AND(P38&lt;&gt;"",Q38&lt;&gt;""),Q38-P38,"")</f>
+        <f>IF(AND(P40&lt;&gt;"",Q40&lt;&gt;""),Q40-P40,"")</f>
         <v/>
       </c>
       <c r="S38" s="13" t="n"/>
@@ -3919,10 +3904,14 @@
     <row r="39" ht="18" customHeight="1" s="31">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>anz</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="n"/>
+          <t>bloomberg</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>analytics &amp; sales</t>
+        </is>
+      </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
           <t>Graduate Program</t>
@@ -3934,7 +3923,9 @@
         </is>
       </c>
       <c r="E39" s="13" t="n"/>
-      <c r="F39" s="13" t="n"/>
+      <c r="F39" s="14" t="n">
+        <v>46266</v>
+      </c>
       <c r="G39" s="13" t="n"/>
       <c r="H39" s="13" t="inlineStr">
         <is>
@@ -3948,15 +3939,27 @@
       <c r="M39" s="13" t="n"/>
       <c r="N39" s="13" t="n"/>
       <c r="O39" s="13" t="n"/>
-      <c r="P39" s="13" t="n"/>
+      <c r="P39" s="14" t="inlineStr">
+        <is>
+          <t>1 Jan 2027-1 Sep 2027</t>
+        </is>
+      </c>
       <c r="Q39" s="17" t="n"/>
       <c r="R39" s="18">
-        <f>IF(AND(P39&lt;&gt;"",Q39&lt;&gt;""),Q39-P39,"")</f>
+        <f>IF(AND(P41&lt;&gt;"",Q41&lt;&gt;""),Q41-P41,"")</f>
         <v/>
       </c>
       <c r="S39" s="13" t="n"/>
-      <c r="T39" s="13" t="n"/>
-      <c r="U39" s="20" t="n"/>
+      <c r="T39" s="13" t="inlineStr">
+        <is>
+          <t>75k-80k</t>
+        </is>
+      </c>
+      <c r="U39" s="20" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
       <c r="V39" s="13" t="n"/>
       <c r="W39" s="13" t="n"/>
       <c r="X39" s="13" t="n"/>
@@ -3969,12 +3972,12 @@
     <row r="40" ht="18" customHeight="1" s="31">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>bcg</t>
+          <t>bmw</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>consulting</t>
+          <t>product</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -3989,7 +3992,7 @@
       </c>
       <c r="E40" s="13" t="n"/>
       <c r="F40" s="14" t="n">
-        <v>46085</v>
+        <v>46117</v>
       </c>
       <c r="G40" s="13" t="n"/>
       <c r="H40" s="13" t="inlineStr">
@@ -4007,7 +4010,7 @@
       <c r="P40" s="13" t="n"/>
       <c r="Q40" s="17" t="n"/>
       <c r="R40" s="18">
-        <f>IF(AND(P40&lt;&gt;"",Q40&lt;&gt;""),Q40-P40,"")</f>
+        <f>IF(AND(P42&lt;&gt;"",Q42&lt;&gt;""),Q42-P42,"")</f>
         <v/>
       </c>
       <c r="S40" s="13" t="n"/>
@@ -4025,17 +4028,17 @@
     <row r="41" ht="18" customHeight="1" s="31">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>bloomberg</t>
+          <t>cisco</t>
         </is>
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>analytics &amp; sales</t>
+          <t>business analyst</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -4044,9 +4047,7 @@
         </is>
       </c>
       <c r="E41" s="13" t="n"/>
-      <c r="F41" s="14" t="n">
-        <v>46266</v>
-      </c>
+      <c r="F41" s="13" t="n"/>
       <c r="G41" s="13" t="n"/>
       <c r="H41" s="13" t="inlineStr">
         <is>
@@ -4060,27 +4061,15 @@
       <c r="M41" s="13" t="n"/>
       <c r="N41" s="13" t="n"/>
       <c r="O41" s="13" t="n"/>
-      <c r="P41" s="14" t="inlineStr">
-        <is>
-          <t>1 Jan 2027-1 Sep 2027</t>
-        </is>
-      </c>
+      <c r="P41" s="13" t="n"/>
       <c r="Q41" s="17" t="n"/>
       <c r="R41" s="18">
-        <f>IF(AND(P41&lt;&gt;"",Q41&lt;&gt;""),Q41-P41,"")</f>
+        <f>IF(AND(P43&lt;&gt;"",Q43&lt;&gt;""),Q43-P43,"")</f>
         <v/>
       </c>
       <c r="S41" s="13" t="n"/>
-      <c r="T41" s="13" t="inlineStr">
-        <is>
-          <t>75k-80k</t>
-        </is>
-      </c>
-      <c r="U41" s="20" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
+      <c r="T41" s="13" t="n"/>
+      <c r="U41" s="20" t="n"/>
       <c r="V41" s="13" t="n"/>
       <c r="W41" s="13" t="n"/>
       <c r="X41" s="13" t="n"/>
@@ -4093,12 +4082,12 @@
     <row r="42" ht="18" customHeight="1" s="31">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>bmw</t>
+          <t>city of gold coast</t>
         </is>
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>product</t>
+          <t>digital and data</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -4108,13 +4097,11 @@
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E42" s="13" t="n"/>
-      <c r="F42" s="14" t="n">
-        <v>46117</v>
-      </c>
+      <c r="F42" s="13" t="n"/>
       <c r="G42" s="13" t="n"/>
       <c r="H42" s="13" t="inlineStr">
         <is>
@@ -4125,13 +4112,17 @@
       <c r="J42" s="13" t="n"/>
       <c r="K42" s="13" t="n"/>
       <c r="L42" s="13" t="n"/>
-      <c r="M42" s="13" t="n"/>
+      <c r="M42" s="13" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
       <c r="N42" s="13" t="n"/>
       <c r="O42" s="13" t="n"/>
       <c r="P42" s="13" t="n"/>
       <c r="Q42" s="17" t="n"/>
       <c r="R42" s="18">
-        <f>IF(AND(P42&lt;&gt;"",Q42&lt;&gt;""),Q42-P42,"")</f>
+        <f>IF(AND(P44&lt;&gt;"",Q44&lt;&gt;""),Q44-P44,"")</f>
         <v/>
       </c>
       <c r="S42" s="13" t="n"/>
@@ -4149,12 +4140,12 @@
     <row r="43" ht="18" customHeight="1" s="31">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>cisco</t>
+          <t>commbank</t>
         </is>
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>business analyst</t>
+          <t>tech ai engineering data science &amp; ai</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -4164,7 +4155,7 @@
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E43" s="13" t="n"/>
@@ -4179,17 +4170,27 @@
       <c r="J43" s="13" t="n"/>
       <c r="K43" s="13" t="n"/>
       <c r="L43" s="13" t="n"/>
-      <c r="M43" s="13" t="n"/>
+      <c r="M43" s="13" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
       <c r="N43" s="13" t="n"/>
       <c r="O43" s="13" t="n"/>
-      <c r="P43" s="13" t="n"/>
+      <c r="P43" s="14" t="n">
+        <v>46349</v>
+      </c>
       <c r="Q43" s="17" t="n"/>
       <c r="R43" s="18">
-        <f>IF(AND(P43&lt;&gt;"",Q43&lt;&gt;""),Q43-P43,"")</f>
+        <f>IF(AND(P45&lt;&gt;"",Q45&lt;&gt;""),Q45-P45,"")</f>
         <v/>
       </c>
       <c r="S43" s="13" t="n"/>
-      <c r="T43" s="13" t="n"/>
+      <c r="T43" s="13" t="inlineStr">
+        <is>
+          <t>65k</t>
+        </is>
+      </c>
       <c r="U43" s="20" t="n"/>
       <c r="V43" s="13" t="n"/>
       <c r="W43" s="13" t="n"/>
@@ -4203,12 +4204,12 @@
     <row r="44" ht="18" customHeight="1" s="31">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>city of gold coast</t>
+          <t>eightcap</t>
         </is>
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>digital and data</t>
+          <t>operations analyst</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
@@ -4218,7 +4219,7 @@
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E44" s="13" t="n"/>
@@ -4243,7 +4244,7 @@
       <c r="P44" s="13" t="n"/>
       <c r="Q44" s="17" t="n"/>
       <c r="R44" s="18">
-        <f>IF(AND(P44&lt;&gt;"",Q44&lt;&gt;""),Q44-P44,"")</f>
+        <f>IF(AND(P48&lt;&gt;"",Q48&lt;&gt;""),Q48-P48,"")</f>
         <v/>
       </c>
       <c r="S44" s="13" t="n"/>
@@ -4261,12 +4262,12 @@
     <row r="45" ht="18" customHeight="1" s="31">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>commbank</t>
+          <t>farrer capital management</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>tech ai engineering data science &amp; ai</t>
+          <t xml:space="preserve">Trade Systems and Operations </t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -4276,11 +4277,13 @@
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E45" s="13" t="n"/>
-      <c r="F45" s="13" t="n"/>
+      <c r="F45" s="14" t="n">
+        <v>46219</v>
+      </c>
       <c r="G45" s="13" t="n"/>
       <c r="H45" s="13" t="inlineStr">
         <is>
@@ -4291,27 +4294,17 @@
       <c r="J45" s="13" t="n"/>
       <c r="K45" s="13" t="n"/>
       <c r="L45" s="13" t="n"/>
-      <c r="M45" s="13" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
+      <c r="M45" s="13" t="n"/>
       <c r="N45" s="13" t="n"/>
       <c r="O45" s="13" t="n"/>
-      <c r="P45" s="14" t="n">
-        <v>46349</v>
-      </c>
+      <c r="P45" s="13" t="n"/>
       <c r="Q45" s="17" t="n"/>
       <c r="R45" s="18">
-        <f>IF(AND(P45&lt;&gt;"",Q45&lt;&gt;""),Q45-P45,"")</f>
+        <f>IF(AND(P49&lt;&gt;"",Q49&lt;&gt;""),Q49-P49,"")</f>
         <v/>
       </c>
       <c r="S45" s="13" t="n"/>
-      <c r="T45" s="13" t="inlineStr">
-        <is>
-          <t>65k</t>
-        </is>
-      </c>
+      <c r="T45" s="13" t="n"/>
       <c r="U45" s="20" t="n"/>
       <c r="V45" s="13" t="n"/>
       <c r="W45" s="13" t="n"/>
@@ -4325,27 +4318,27 @@
     <row r="46" ht="17.25" customHeight="1" s="31">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>digital graduate program gov</t>
+          <t>fivecast</t>
         </is>
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>data analyst</t>
+          <t>data science</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E46" s="13" t="n"/>
       <c r="F46" s="14" t="n">
-        <v>46278</v>
+        <v>46169</v>
       </c>
       <c r="G46" s="13" t="n"/>
       <c r="H46" s="13" t="inlineStr">
@@ -4357,27 +4350,17 @@
       <c r="J46" s="13" t="n"/>
       <c r="K46" s="13" t="n"/>
       <c r="L46" s="13" t="n"/>
-      <c r="M46" s="13" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
+      <c r="M46" s="13" t="n"/>
       <c r="N46" s="13" t="n"/>
       <c r="O46" s="13" t="n"/>
-      <c r="P46" s="14" t="n">
-        <v>46054</v>
-      </c>
+      <c r="P46" s="13" t="n"/>
       <c r="Q46" s="17" t="n"/>
       <c r="R46" s="18">
-        <f>IF(AND(P46&lt;&gt;"",Q46&lt;&gt;""),Q46-P46,"")</f>
+        <f>IF(AND(P50&lt;&gt;"",Q50&lt;&gt;""),Q50-P50,"")</f>
         <v/>
       </c>
       <c r="S46" s="13" t="n"/>
-      <c r="T46" s="13" t="inlineStr">
-        <is>
-          <t>77-84k</t>
-        </is>
-      </c>
+      <c r="T46" s="13" t="n"/>
       <c r="U46" s="20" t="n"/>
       <c r="V46" s="13" t="n"/>
       <c r="W46" s="13" t="n"/>
@@ -4391,22 +4374,26 @@
     <row r="47" ht="18" customHeight="1" s="31">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>disney</t>
+          <t>flight centre</t>
         </is>
       </c>
       <c r="B47" s="13" t="n"/>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E47" s="13" t="n"/>
-      <c r="F47" s="13" t="n"/>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>sep</t>
+        </is>
+      </c>
       <c r="G47" s="13" t="n"/>
       <c r="H47" s="13" t="inlineStr">
         <is>
@@ -4417,17 +4404,13 @@
       <c r="J47" s="13" t="n"/>
       <c r="K47" s="13" t="n"/>
       <c r="L47" s="13" t="n"/>
-      <c r="M47" s="13" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
+      <c r="M47" s="13" t="n"/>
       <c r="N47" s="13" t="n"/>
       <c r="O47" s="13" t="n"/>
       <c r="P47" s="13" t="n"/>
       <c r="Q47" s="17" t="n"/>
       <c r="R47" s="18">
-        <f>IF(AND(P47&lt;&gt;"",Q47&lt;&gt;""),Q47-P47,"")</f>
+        <f>IF(AND(P51&lt;&gt;"",Q51&lt;&gt;""),Q51-P51,"")</f>
         <v/>
       </c>
       <c r="S47" s="13" t="n"/>
@@ -4445,26 +4428,28 @@
     <row r="48" ht="18" customHeight="1" s="31">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>eightcap</t>
+          <t>FTI Consulting</t>
         </is>
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>operations analyst</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>NSW, WA</t>
         </is>
       </c>
       <c r="E48" s="13" t="n"/>
-      <c r="F48" s="13" t="n"/>
+      <c r="F48" s="14" t="n">
+        <v>46093</v>
+      </c>
       <c r="G48" s="13" t="n"/>
       <c r="H48" s="13" t="inlineStr">
         <is>
@@ -4475,22 +4460,30 @@
       <c r="J48" s="13" t="n"/>
       <c r="K48" s="13" t="n"/>
       <c r="L48" s="13" t="n"/>
-      <c r="M48" s="13" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
+      <c r="M48" s="13" t="n"/>
       <c r="N48" s="13" t="n"/>
       <c r="O48" s="13" t="n"/>
-      <c r="P48" s="13" t="n"/>
+      <c r="P48" s="14" t="inlineStr">
+        <is>
+          <t>4 May 2026 - 18 Jul 2026</t>
+        </is>
+      </c>
       <c r="Q48" s="17" t="n"/>
       <c r="R48" s="18">
-        <f>IF(AND(P48&lt;&gt;"",Q48&lt;&gt;""),Q48-P48,"")</f>
+        <f>IF(AND(P52&lt;&gt;"",Q52&lt;&gt;""),Q52-P52,"")</f>
         <v/>
       </c>
       <c r="S48" s="13" t="n"/>
-      <c r="T48" s="13" t="n"/>
-      <c r="U48" s="20" t="n"/>
+      <c r="T48" s="13" t="inlineStr">
+        <is>
+          <t>36 / Hour</t>
+        </is>
+      </c>
+      <c r="U48" s="20" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
       <c r="V48" s="13" t="n"/>
       <c r="W48" s="13" t="n"/>
       <c r="X48" s="13" t="n"/>
@@ -4503,17 +4496,17 @@
     <row r="49" ht="15.75" customHeight="1" s="31">
       <c r="A49" s="13" t="inlineStr">
         <is>
-          <t>farrer capital management</t>
+          <t>fujitsu</t>
         </is>
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trade Systems and Operations </t>
+          <t>Business Analyst</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D49" s="13" t="inlineStr">
@@ -4522,8 +4515,10 @@
         </is>
       </c>
       <c r="E49" s="13" t="n"/>
-      <c r="F49" s="14" t="n">
-        <v>46219</v>
+      <c r="F49" s="23" t="inlineStr">
+        <is>
+          <t>sep</t>
+        </is>
       </c>
       <c r="G49" s="13" t="n"/>
       <c r="H49" s="13" t="inlineStr">
@@ -4541,7 +4536,7 @@
       <c r="P49" s="13" t="n"/>
       <c r="Q49" s="17" t="n"/>
       <c r="R49" s="18">
-        <f>IF(AND(P49&lt;&gt;"",Q49&lt;&gt;""),Q49-P49,"")</f>
+        <f>IF(AND(P53&lt;&gt;"",Q53&lt;&gt;""),Q53-P53,"")</f>
         <v/>
       </c>
       <c r="S49" s="13" t="n"/>
@@ -4557,17 +4552,17 @@
       <c r="AC49" s="13" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="31">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>fivecast</t>
-        </is>
-      </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>data science</t>
-        </is>
-      </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>general motors</t>
+        </is>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>Service Operations Business</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
@@ -4578,8 +4573,10 @@
         </is>
       </c>
       <c r="E50" s="13" t="n"/>
-      <c r="F50" s="14" t="n">
-        <v>46169</v>
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>oct</t>
+        </is>
       </c>
       <c r="G50" s="13" t="n"/>
       <c r="H50" s="13" t="inlineStr">
@@ -4597,7 +4594,7 @@
       <c r="P50" s="13" t="n"/>
       <c r="Q50" s="17" t="n"/>
       <c r="R50" s="18">
-        <f>IF(AND(P50&lt;&gt;"",Q50&lt;&gt;""),Q50-P50,"")</f>
+        <f>IF(AND(P54&lt;&gt;"",Q54&lt;&gt;""),Q54-P54,"")</f>
         <v/>
       </c>
       <c r="S50" s="13" t="n"/>
@@ -4615,10 +4612,14 @@
     <row r="51" ht="15.75" customHeight="1" s="31">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>flight centre</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="n"/>
+          <t>hatch</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Analyst - Advisory</t>
+        </is>
+      </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
           <t>Graduate Program</t>
@@ -4630,11 +4631,7 @@
         </is>
       </c>
       <c r="E51" s="13" t="n"/>
-      <c r="F51" s="14" t="inlineStr">
-        <is>
-          <t>sep</t>
-        </is>
-      </c>
+      <c r="F51" s="13" t="n"/>
       <c r="G51" s="13" t="n"/>
       <c r="H51" s="13" t="inlineStr">
         <is>
@@ -4651,7 +4648,7 @@
       <c r="P51" s="13" t="n"/>
       <c r="Q51" s="17" t="n"/>
       <c r="R51" s="18">
-        <f>IF(AND(P51&lt;&gt;"",Q51&lt;&gt;""),Q51-P51,"")</f>
+        <f>IF(AND(P55&lt;&gt;"",Q55&lt;&gt;""),Q55-P55,"")</f>
         <v/>
       </c>
       <c r="S51" s="13" t="n"/>
@@ -4669,12 +4666,12 @@
     <row r="52" ht="15.75" customHeight="1" s="31">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>FTI Consulting</t>
+          <t>Heidi Health</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
         <is>
-          <t>Data Analytics</t>
+          <t>Strategy &amp; Data Intern</t>
         </is>
       </c>
       <c r="C52" s="13" t="inlineStr">
@@ -4684,13 +4681,11 @@
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>NSW, WA</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E52" s="13" t="n"/>
-      <c r="F52" s="14" t="n">
-        <v>46093</v>
-      </c>
+      <c r="F52" s="13" t="n"/>
       <c r="G52" s="13" t="n"/>
       <c r="H52" s="13" t="inlineStr">
         <is>
@@ -4704,27 +4699,17 @@
       <c r="M52" s="13" t="n"/>
       <c r="N52" s="13" t="n"/>
       <c r="O52" s="13" t="n"/>
-      <c r="P52" s="14" t="inlineStr">
-        <is>
-          <t>4 May 2026 - 18 Jul 2026</t>
-        </is>
+      <c r="P52" s="14" t="n">
+        <v>46124</v>
       </c>
       <c r="Q52" s="17" t="n"/>
       <c r="R52" s="18">
-        <f>IF(AND(P52&lt;&gt;"",Q52&lt;&gt;""),Q52-P52,"")</f>
+        <f>IF(AND(P56&lt;&gt;"",Q56&lt;&gt;""),Q56-P56,"")</f>
         <v/>
       </c>
       <c r="S52" s="13" t="n"/>
-      <c r="T52" s="13" t="inlineStr">
-        <is>
-          <t>36 / Hour</t>
-        </is>
-      </c>
-      <c r="U52" s="20" t="inlineStr">
-        <is>
-          <t>2-4</t>
-        </is>
-      </c>
+      <c r="T52" s="13" t="n"/>
+      <c r="U52" s="20" t="n"/>
       <c r="V52" s="13" t="n"/>
       <c r="W52" s="13" t="n"/>
       <c r="X52" s="13" t="n"/>
@@ -4737,17 +4722,17 @@
     <row r="53" ht="15.75" customHeight="1" s="31">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>fujitsu</t>
+          <t>IMC</t>
         </is>
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>Business Analyst</t>
+          <t>quantitative research</t>
         </is>
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
@@ -4756,10 +4741,8 @@
         </is>
       </c>
       <c r="E53" s="13" t="n"/>
-      <c r="F53" s="23" t="inlineStr">
-        <is>
-          <t>sep</t>
-        </is>
+      <c r="F53" s="14" t="n">
+        <v>46203</v>
       </c>
       <c r="G53" s="13" t="n"/>
       <c r="H53" s="13" t="inlineStr">
@@ -4777,7 +4760,7 @@
       <c r="P53" s="13" t="n"/>
       <c r="Q53" s="17" t="n"/>
       <c r="R53" s="18">
-        <f>IF(AND(P53&lt;&gt;"",Q53&lt;&gt;""),Q53-P53,"")</f>
+        <f>IF(AND(P57&lt;&gt;"",Q57&lt;&gt;""),Q57-P57,"")</f>
         <v/>
       </c>
       <c r="S53" s="13" t="n"/>
@@ -4793,19 +4776,19 @@
       <c r="AC53" s="13" t="n"/>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="31">
-      <c r="A54" s="21" t="inlineStr">
-        <is>
-          <t>general motors</t>
-        </is>
-      </c>
-      <c r="B54" s="21" t="inlineStr">
-        <is>
-          <t>Service Operations Business</t>
-        </is>
-      </c>
-      <c r="C54" s="21" t="inlineStr">
-        <is>
-          <t>Internship</t>
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>jpmorganchase</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>coporate analyst</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
@@ -4814,10 +4797,8 @@
         </is>
       </c>
       <c r="E54" s="13" t="n"/>
-      <c r="F54" s="23" t="inlineStr">
-        <is>
-          <t>oct</t>
-        </is>
+      <c r="F54" s="14" t="n">
+        <v>46108</v>
       </c>
       <c r="G54" s="13" t="n"/>
       <c r="H54" s="13" t="inlineStr">
@@ -4835,7 +4816,7 @@
       <c r="P54" s="13" t="n"/>
       <c r="Q54" s="17" t="n"/>
       <c r="R54" s="18">
-        <f>IF(AND(P54&lt;&gt;"",Q54&lt;&gt;""),Q54-P54,"")</f>
+        <f>IF(AND(P58&lt;&gt;"",Q58&lt;&gt;""),Q58-P58,"")</f>
         <v/>
       </c>
       <c r="S54" s="13" t="n"/>
@@ -4853,12 +4834,12 @@
     <row r="55" ht="15.75" customHeight="1" s="31">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>hatch</t>
+          <t>KPMG</t>
         </is>
       </c>
       <c r="B55" s="13" t="inlineStr">
         <is>
-          <t>Analyst - Advisory</t>
+          <t>Forensic Risk - Consulting</t>
         </is>
       </c>
       <c r="C55" s="13" t="inlineStr">
@@ -4868,11 +4849,13 @@
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E55" s="13" t="n"/>
-      <c r="F55" s="13" t="n"/>
+      <c r="F55" s="14" t="n">
+        <v>46091</v>
+      </c>
       <c r="G55" s="13" t="n"/>
       <c r="H55" s="13" t="inlineStr">
         <is>
@@ -4886,15 +4869,25 @@
       <c r="M55" s="13" t="n"/>
       <c r="N55" s="13" t="n"/>
       <c r="O55" s="13" t="n"/>
-      <c r="P55" s="13" t="n"/>
+      <c r="P55" s="14" t="n">
+        <v>46426</v>
+      </c>
       <c r="Q55" s="17" t="n"/>
       <c r="R55" s="18">
-        <f>IF(AND(P55&lt;&gt;"",Q55&lt;&gt;""),Q55-P55,"")</f>
+        <f>IF(AND(P59&lt;&gt;"",Q59&lt;&gt;""),Q59-P59,"")</f>
         <v/>
       </c>
       <c r="S55" s="13" t="n"/>
-      <c r="T55" s="13" t="n"/>
-      <c r="U55" s="20" t="n"/>
+      <c r="T55" s="13" t="inlineStr">
+        <is>
+          <t>60k-82k</t>
+        </is>
+      </c>
+      <c r="U55" s="20" t="inlineStr">
+        <is>
+          <t>1-700</t>
+        </is>
+      </c>
       <c r="V55" s="13" t="n"/>
       <c r="W55" s="13" t="n"/>
       <c r="X55" s="13" t="n"/>
@@ -4907,17 +4900,17 @@
     <row r="56" ht="15.75" customHeight="1" s="31">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>Heidi Health</t>
+          <t>loreal</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
         <is>
-          <t>Strategy &amp; Data Intern</t>
+          <t>Management Trainee Program – Data &amp; Analytics Stream</t>
         </is>
       </c>
       <c r="C56" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D56" s="13" t="inlineStr">
@@ -4926,8 +4919,12 @@
         </is>
       </c>
       <c r="E56" s="13" t="n"/>
-      <c r="F56" s="13" t="n"/>
-      <c r="G56" s="13" t="n"/>
+      <c r="F56" s="14" t="n">
+        <v>46093</v>
+      </c>
+      <c r="G56" s="33" t="n">
+        <v>46277</v>
+      </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -4937,20 +4934,32 @@
       <c r="J56" s="13" t="n"/>
       <c r="K56" s="13" t="n"/>
       <c r="L56" s="13" t="n"/>
-      <c r="M56" s="13" t="n"/>
+      <c r="M56" s="13" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
       <c r="N56" s="13" t="n"/>
       <c r="O56" s="13" t="n"/>
       <c r="P56" s="14" t="n">
-        <v>46124</v>
+        <v>46416</v>
       </c>
       <c r="Q56" s="17" t="n"/>
       <c r="R56" s="18">
-        <f>IF(AND(P56&lt;&gt;"",Q56&lt;&gt;""),Q56-P56,"")</f>
+        <f>IF(AND(P60&lt;&gt;"",Q60&lt;&gt;""),Q60-P60,"")</f>
         <v/>
       </c>
       <c r="S56" s="13" t="n"/>
-      <c r="T56" s="13" t="n"/>
-      <c r="U56" s="20" t="n"/>
+      <c r="T56" s="13" t="inlineStr">
+        <is>
+          <t>66k-75k</t>
+        </is>
+      </c>
+      <c r="U56" s="20" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
       <c r="V56" s="13" t="n"/>
       <c r="W56" s="13" t="n"/>
       <c r="X56" s="13" t="n"/>
@@ -4963,27 +4972,27 @@
     <row r="57" ht="15.75" customHeight="1" s="31">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>IMC</t>
+          <t>McGrathNicol</t>
         </is>
       </c>
       <c r="B57" s="13" t="inlineStr">
         <is>
-          <t>quantitative research</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E57" s="13" t="n"/>
       <c r="F57" s="14" t="n">
-        <v>46203</v>
+        <v>46264</v>
       </c>
       <c r="G57" s="13" t="n"/>
       <c r="H57" s="13" t="inlineStr">
@@ -4998,15 +5007,25 @@
       <c r="M57" s="13" t="n"/>
       <c r="N57" s="13" t="n"/>
       <c r="O57" s="13" t="n"/>
-      <c r="P57" s="13" t="n"/>
+      <c r="P57" s="14" t="n">
+        <v>46440</v>
+      </c>
       <c r="Q57" s="17" t="n"/>
       <c r="R57" s="18">
-        <f>IF(AND(P57&lt;&gt;"",Q57&lt;&gt;""),Q57-P57,"")</f>
+        <f>IF(AND(P61&lt;&gt;"",Q61&lt;&gt;""),Q61-P61,"")</f>
         <v/>
       </c>
       <c r="S57" s="13" t="n"/>
-      <c r="T57" s="13" t="n"/>
-      <c r="U57" s="20" t="n"/>
+      <c r="T57" s="13" t="inlineStr">
+        <is>
+          <t>78k</t>
+        </is>
+      </c>
+      <c r="U57" s="20" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
       <c r="V57" s="13" t="n"/>
       <c r="W57" s="13" t="n"/>
       <c r="X57" s="13" t="n"/>
@@ -5019,12 +5038,12 @@
     <row r="58" ht="15.75" customHeight="1" s="31">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>jpmorganchase</t>
+          <t>mckinsey &amp; company</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
         <is>
-          <t>coporate analyst</t>
+          <t>business analsyt</t>
         </is>
       </c>
       <c r="C58" s="13" t="inlineStr">
@@ -5039,7 +5058,7 @@
       </c>
       <c r="E58" s="13" t="n"/>
       <c r="F58" s="14" t="n">
-        <v>46108</v>
+        <v>46075</v>
       </c>
       <c r="G58" s="13" t="n"/>
       <c r="H58" s="13" t="inlineStr">
@@ -5057,7 +5076,7 @@
       <c r="P58" s="13" t="n"/>
       <c r="Q58" s="17" t="n"/>
       <c r="R58" s="18">
-        <f>IF(AND(P58&lt;&gt;"",Q58&lt;&gt;""),Q58-P58,"")</f>
+        <f>IF(AND(P62&lt;&gt;"",Q62&lt;&gt;""),Q62-P62,"")</f>
         <v/>
       </c>
       <c r="S58" s="13" t="n"/>
@@ -5075,27 +5094,29 @@
     <row r="59" ht="15.75" customHeight="1" s="31">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>KPMG</t>
+          <t>mercedes benz</t>
         </is>
       </c>
       <c r="B59" s="13" t="inlineStr">
         <is>
-          <t>Forensic Risk - Consulting</t>
+          <t>performance &amp; Insights</t>
         </is>
       </c>
       <c r="C59" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D59" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E59" s="13" t="n"/>
-      <c r="F59" s="14" t="n">
-        <v>46091</v>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>oct</t>
+        </is>
       </c>
       <c r="G59" s="13" t="n"/>
       <c r="H59" s="13" t="inlineStr">
@@ -5110,25 +5131,15 @@
       <c r="M59" s="13" t="n"/>
       <c r="N59" s="13" t="n"/>
       <c r="O59" s="13" t="n"/>
-      <c r="P59" s="14" t="n">
-        <v>46426</v>
-      </c>
+      <c r="P59" s="13" t="n"/>
       <c r="Q59" s="17" t="n"/>
       <c r="R59" s="18">
-        <f>IF(AND(P59&lt;&gt;"",Q59&lt;&gt;""),Q59-P59,"")</f>
+        <f>IF(AND(P63&lt;&gt;"",Q63&lt;&gt;""),Q63-P63,"")</f>
         <v/>
       </c>
       <c r="S59" s="13" t="n"/>
-      <c r="T59" s="13" t="inlineStr">
-        <is>
-          <t>60k-82k</t>
-        </is>
-      </c>
-      <c r="U59" s="20" t="inlineStr">
-        <is>
-          <t>1-700</t>
-        </is>
-      </c>
+      <c r="T59" s="13" t="n"/>
+      <c r="U59" s="20" t="n"/>
       <c r="V59" s="13" t="n"/>
       <c r="W59" s="13" t="n"/>
       <c r="X59" s="13" t="n"/>
@@ -5141,27 +5152,27 @@
     <row r="60" ht="15.75" customHeight="1" s="31">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>loreal</t>
+          <t>moody's corporation</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
         <is>
-          <t>Management Trainee Program – Data &amp; Analytics Stream</t>
+          <t>Predictive Analytics Intern</t>
         </is>
       </c>
       <c r="C60" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E60" s="13" t="n"/>
       <c r="F60" s="14" t="n">
-        <v>46093</v>
+        <v>46140</v>
       </c>
       <c r="G60" s="13" t="n"/>
       <c r="H60" s="13" t="inlineStr">
@@ -5176,25 +5187,15 @@
       <c r="M60" s="13" t="n"/>
       <c r="N60" s="13" t="n"/>
       <c r="O60" s="13" t="n"/>
-      <c r="P60" s="14" t="n">
-        <v>46416</v>
-      </c>
+      <c r="P60" s="13" t="n"/>
       <c r="Q60" s="17" t="n"/>
       <c r="R60" s="18">
-        <f>IF(AND(P60&lt;&gt;"",Q60&lt;&gt;""),Q60-P60,"")</f>
+        <f>IF(AND(P64&lt;&gt;"",Q64&lt;&gt;""),Q64-P64,"")</f>
         <v/>
       </c>
       <c r="S60" s="13" t="n"/>
-      <c r="T60" s="13" t="inlineStr">
-        <is>
-          <t>66k-75k</t>
-        </is>
-      </c>
-      <c r="U60" s="20" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
+      <c r="T60" s="13" t="n"/>
+      <c r="U60" s="20" t="n"/>
       <c r="V60" s="13" t="n"/>
       <c r="W60" s="13" t="n"/>
       <c r="X60" s="13" t="n"/>
@@ -5207,27 +5208,27 @@
     <row r="61" ht="15.75" customHeight="1" s="31">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>McGrathNicol</t>
+          <t>nab</t>
         </is>
       </c>
       <c r="B61" s="13" t="inlineStr">
         <is>
-          <t>Data Analytics</t>
+          <t>digital data and ai</t>
         </is>
       </c>
       <c r="C61" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D61" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E61" s="13" t="n"/>
       <c r="F61" s="14" t="n">
-        <v>46264</v>
+        <v>46243</v>
       </c>
       <c r="G61" s="13" t="n"/>
       <c r="H61" s="13" t="inlineStr">
@@ -5243,44 +5244,44 @@
       <c r="N61" s="13" t="n"/>
       <c r="O61" s="13" t="n"/>
       <c r="P61" s="14" t="n">
-        <v>46440</v>
+        <v>46349</v>
       </c>
       <c r="Q61" s="17" t="n"/>
       <c r="R61" s="18">
-        <f>IF(AND(P61&lt;&gt;"",Q61&lt;&gt;""),Q61-P61,"")</f>
+        <f>IF(AND(P65&lt;&gt;"",Q65&lt;&gt;""),Q65-P65,"")</f>
         <v/>
       </c>
       <c r="S61" s="13" t="n"/>
       <c r="T61" s="13" t="inlineStr">
         <is>
-          <t>78k</t>
-        </is>
-      </c>
-      <c r="U61" s="20" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
+          <t>65-70k</t>
+        </is>
+      </c>
+      <c r="U61" s="20" t="n"/>
       <c r="V61" s="13" t="n"/>
       <c r="W61" s="13" t="n"/>
       <c r="X61" s="13" t="n"/>
       <c r="Y61" s="13" t="n"/>
       <c r="Z61" s="13" t="n"/>
-      <c r="AA61" s="13" t="n"/>
-      <c r="AB61" s="13" t="n"/>
+      <c r="AA61" s="13" t="inlineStr">
+        <is>
+          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
+        </is>
+      </c>
+      <c r="AB61" s="13" t="inlineStr">
+        <is>
+          <t>Insurance Risk &amp; Claims Analytics Dashboard, Bank Loan Application Tracking Dashboard, Credit Fraud Detection Classifier Analysis, Customer Segmentation in Bank Campaigns Presentation</t>
+        </is>
+      </c>
       <c r="AC61" s="13" t="n"/>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="31">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>mckinsey &amp; company</t>
-        </is>
-      </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>business analsyt</t>
-        </is>
-      </c>
+          <t>nestle</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="n"/>
       <c r="C62" s="13" t="inlineStr">
         <is>
           <t>Graduate Program</t>
@@ -5292,8 +5293,10 @@
         </is>
       </c>
       <c r="E62" s="13" t="n"/>
-      <c r="F62" s="14" t="n">
-        <v>46075</v>
+      <c r="F62" s="14" t="inlineStr">
+        <is>
+          <t>june</t>
+        </is>
       </c>
       <c r="G62" s="13" t="n"/>
       <c r="H62" s="13" t="inlineStr">
@@ -5311,7 +5314,7 @@
       <c r="P62" s="13" t="n"/>
       <c r="Q62" s="17" t="n"/>
       <c r="R62" s="18">
-        <f>IF(AND(P62&lt;&gt;"",Q62&lt;&gt;""),Q62-P62,"")</f>
+        <f>IF(AND(P66&lt;&gt;"",Q66&lt;&gt;""),Q66-P66,"")</f>
         <v/>
       </c>
       <c r="S62" s="13" t="n"/>
@@ -5329,17 +5332,17 @@
     <row r="63" ht="15.75" customHeight="1" s="31">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>mercedes benz</t>
+          <t>NSW government</t>
         </is>
       </c>
       <c r="B63" s="13" t="inlineStr">
         <is>
-          <t>performance &amp; Insights</t>
+          <t>Data analytics</t>
         </is>
       </c>
       <c r="C63" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D63" s="13" t="inlineStr">
@@ -5348,11 +5351,7 @@
         </is>
       </c>
       <c r="E63" s="13" t="n"/>
-      <c r="F63" s="14" t="inlineStr">
-        <is>
-          <t>oct</t>
-        </is>
-      </c>
+      <c r="F63" s="13" t="n"/>
       <c r="G63" s="13" t="n"/>
       <c r="H63" s="13" t="inlineStr">
         <is>
@@ -5369,7 +5368,7 @@
       <c r="P63" s="13" t="n"/>
       <c r="Q63" s="17" t="n"/>
       <c r="R63" s="18">
-        <f>IF(AND(P63&lt;&gt;"",Q63&lt;&gt;""),Q63-P63,"")</f>
+        <f>IF(AND(P67&lt;&gt;"",Q67&lt;&gt;""),Q67-P67,"")</f>
         <v/>
       </c>
       <c r="S63" s="13" t="n"/>
@@ -5387,17 +5386,17 @@
     <row r="64" ht="15.75" customHeight="1" s="31">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>moody's corporation</t>
+          <t>nti</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
         <is>
-          <t>Predictive Analytics Intern</t>
+          <t xml:space="preserve">Graduate Business Analyst - IT </t>
         </is>
       </c>
       <c r="C64" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
@@ -5406,8 +5405,10 @@
         </is>
       </c>
       <c r="E64" s="13" t="n"/>
-      <c r="F64" s="14" t="n">
-        <v>46140</v>
+      <c r="F64" s="14" t="inlineStr">
+        <is>
+          <t>jun</t>
+        </is>
       </c>
       <c r="G64" s="13" t="n"/>
       <c r="H64" s="13" t="inlineStr">
@@ -5425,7 +5426,7 @@
       <c r="P64" s="13" t="n"/>
       <c r="Q64" s="17" t="n"/>
       <c r="R64" s="18">
-        <f>IF(AND(P64&lt;&gt;"",Q64&lt;&gt;""),Q64-P64,"")</f>
+        <f>IF(AND(P68&lt;&gt;"",Q68&lt;&gt;""),Q68-P68,"")</f>
         <v/>
       </c>
       <c r="S64" s="13" t="n"/>
@@ -5443,12 +5444,12 @@
     <row r="65" ht="15.75" customHeight="1" s="31">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>nab</t>
+          <t>openmesh</t>
         </is>
       </c>
       <c r="B65" s="13" t="inlineStr">
         <is>
-          <t>digital data and ai</t>
+          <t>data science or analyst</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
@@ -5458,12 +5459,14 @@
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E65" s="13" t="n"/>
-      <c r="F65" s="14" t="n">
-        <v>46243</v>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>oct</t>
+        </is>
       </c>
       <c r="G65" s="13" t="n"/>
       <c r="H65" s="13" t="inlineStr">
@@ -5478,45 +5481,35 @@
       <c r="M65" s="13" t="n"/>
       <c r="N65" s="13" t="n"/>
       <c r="O65" s="13" t="n"/>
-      <c r="P65" s="14" t="n">
-        <v>46349</v>
-      </c>
+      <c r="P65" s="13" t="n"/>
       <c r="Q65" s="17" t="n"/>
       <c r="R65" s="18">
-        <f>IF(AND(P65&lt;&gt;"",Q65&lt;&gt;""),Q65-P65,"")</f>
+        <f>IF(AND(P69&lt;&gt;"",Q69&lt;&gt;""),Q69-P69,"")</f>
         <v/>
       </c>
       <c r="S65" s="13" t="n"/>
-      <c r="T65" s="13" t="inlineStr">
-        <is>
-          <t>65-70k</t>
-        </is>
-      </c>
+      <c r="T65" s="13" t="n"/>
       <c r="U65" s="20" t="n"/>
       <c r="V65" s="13" t="n"/>
       <c r="W65" s="13" t="n"/>
       <c r="X65" s="13" t="n"/>
       <c r="Y65" s="13" t="n"/>
       <c r="Z65" s="13" t="n"/>
-      <c r="AA65" s="13" t="inlineStr">
-        <is>
-          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
-        </is>
-      </c>
-      <c r="AB65" s="13" t="inlineStr">
-        <is>
-          <t>Insurance Risk &amp; Claims Analytics Dashboard, Bank Loan Application Tracking Dashboard, Credit Fraud Detection Classifier Analysis, Customer Segmentation in Bank Campaigns Presentation</t>
-        </is>
-      </c>
+      <c r="AA65" s="13" t="n"/>
+      <c r="AB65" s="13" t="n"/>
       <c r="AC65" s="13" t="n"/>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="31">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>nestle</t>
-        </is>
-      </c>
-      <c r="B66" s="13" t="n"/>
+          <t>optiver</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>quantitative research</t>
+        </is>
+      </c>
       <c r="C66" s="13" t="inlineStr">
         <is>
           <t>Graduate Program</t>
@@ -5528,10 +5521,8 @@
         </is>
       </c>
       <c r="E66" s="13" t="n"/>
-      <c r="F66" s="14" t="inlineStr">
-        <is>
-          <t>june</t>
-        </is>
+      <c r="F66" s="14" t="n">
+        <v>46122</v>
       </c>
       <c r="G66" s="13" t="n"/>
       <c r="H66" s="13" t="inlineStr">
@@ -5549,7 +5540,7 @@
       <c r="P66" s="13" t="n"/>
       <c r="Q66" s="17" t="n"/>
       <c r="R66" s="18">
-        <f>IF(AND(P66&lt;&gt;"",Q66&lt;&gt;""),Q66-P66,"")</f>
+        <f>IF(AND(P70&lt;&gt;"",Q70&lt;&gt;""),Q70-P70,"")</f>
         <v/>
       </c>
       <c r="S66" s="13" t="n"/>
@@ -5567,12 +5558,12 @@
     <row r="67" ht="15.75" customHeight="1" s="31">
       <c r="A67" s="13" t="inlineStr">
         <is>
-          <t>NSW government</t>
+          <t>origin</t>
         </is>
       </c>
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>Data analytics</t>
+          <t>business analyst</t>
         </is>
       </c>
       <c r="C67" s="13" t="inlineStr">
@@ -5586,8 +5577,12 @@
         </is>
       </c>
       <c r="E67" s="13" t="n"/>
-      <c r="F67" s="13" t="n"/>
-      <c r="G67" s="13" t="n"/>
+      <c r="F67" s="14" t="n">
+        <v>46166</v>
+      </c>
+      <c r="G67" s="14" t="n">
+        <v>46166</v>
+      </c>
       <c r="H67" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -5603,7 +5598,7 @@
       <c r="P67" s="13" t="n"/>
       <c r="Q67" s="17" t="n"/>
       <c r="R67" s="18">
-        <f>IF(AND(P67&lt;&gt;"",Q67&lt;&gt;""),Q67-P67,"")</f>
+        <f>IF(AND(P71&lt;&gt;"",Q71&lt;&gt;""),Q71-P71,"")</f>
         <v/>
       </c>
       <c r="S67" s="13" t="n"/>
@@ -5614,24 +5609,32 @@
       <c r="X67" s="13" t="n"/>
       <c r="Y67" s="13" t="n"/>
       <c r="Z67" s="13" t="n"/>
-      <c r="AA67" s="13" t="n"/>
-      <c r="AB67" s="13" t="n"/>
+      <c r="AA67" s="13" t="inlineStr">
+        <is>
+          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
+        </is>
+      </c>
+      <c r="AB67" s="13" t="inlineStr">
+        <is>
+          <t>Customer Churn Forecasting Analysis in Telecom Services, Insurance Risk &amp; Claims Analytics Dashboard, Vendor Performance Analytics Dashboard, Credit Fraud Detection Classifier Analysis</t>
+        </is>
+      </c>
       <c r="AC67" s="13" t="n"/>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="31">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>nti</t>
+          <t>QBE Insurance</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graduate Business Analyst - IT </t>
+          <t>data analytics</t>
         </is>
       </c>
       <c r="C68" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D68" s="13" t="inlineStr">
@@ -5640,10 +5643,8 @@
         </is>
       </c>
       <c r="E68" s="13" t="n"/>
-      <c r="F68" s="14" t="inlineStr">
-        <is>
-          <t>jun</t>
-        </is>
+      <c r="F68" s="14" t="n">
+        <v>46253</v>
       </c>
       <c r="G68" s="13" t="n"/>
       <c r="H68" s="13" t="inlineStr">
@@ -5661,7 +5662,7 @@
       <c r="P68" s="13" t="n"/>
       <c r="Q68" s="17" t="n"/>
       <c r="R68" s="18">
-        <f>IF(AND(P68&lt;&gt;"",Q68&lt;&gt;""),Q68-P68,"")</f>
+        <f>IF(AND(P72&lt;&gt;"",Q72&lt;&gt;""),Q72-P72,"")</f>
         <v/>
       </c>
       <c r="S68" s="13" t="n"/>
@@ -5679,30 +5680,26 @@
     <row r="69" ht="15.75" customHeight="1" s="31">
       <c r="A69" s="13" t="inlineStr">
         <is>
-          <t>openmesh</t>
+          <t xml:space="preserve">queensland government digital </t>
         </is>
       </c>
       <c r="B69" s="13" t="inlineStr">
         <is>
-          <t>data science or analyst</t>
+          <t>Data analytics</t>
         </is>
       </c>
       <c r="C69" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate School</t>
         </is>
       </c>
       <c r="D69" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E69" s="13" t="n"/>
-      <c r="F69" s="14" t="inlineStr">
-        <is>
-          <t>oct</t>
-        </is>
-      </c>
+      <c r="F69" s="13" t="n"/>
       <c r="G69" s="13" t="n"/>
       <c r="H69" s="13" t="inlineStr">
         <is>
@@ -5719,7 +5716,7 @@
       <c r="P69" s="13" t="n"/>
       <c r="Q69" s="17" t="n"/>
       <c r="R69" s="18">
-        <f>IF(AND(P69&lt;&gt;"",Q69&lt;&gt;""),Q69-P69,"")</f>
+        <f>IF(AND(P73&lt;&gt;"",Q73&lt;&gt;""),Q73-P73,"")</f>
         <v/>
       </c>
       <c r="S69" s="13" t="n"/>
@@ -5737,12 +5734,12 @@
     <row r="70" ht="15.75" customHeight="1" s="31">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>optiver</t>
+          <t>shell</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
         <is>
-          <t>quantitative research</t>
+          <t>business analyst</t>
         </is>
       </c>
       <c r="C70" s="13" t="inlineStr">
@@ -5756,8 +5753,10 @@
         </is>
       </c>
       <c r="E70" s="13" t="n"/>
-      <c r="F70" s="14" t="n">
-        <v>46122</v>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t>sep</t>
+        </is>
       </c>
       <c r="G70" s="13" t="n"/>
       <c r="H70" s="13" t="inlineStr">
@@ -5775,7 +5774,7 @@
       <c r="P70" s="13" t="n"/>
       <c r="Q70" s="17" t="n"/>
       <c r="R70" s="18">
-        <f>IF(AND(P70&lt;&gt;"",Q70&lt;&gt;""),Q70-P70,"")</f>
+        <f>IF(AND(P74&lt;&gt;"",Q74&lt;&gt;""),Q74-P74,"")</f>
         <v/>
       </c>
       <c r="S70" s="13" t="n"/>
@@ -5793,12 +5792,12 @@
     <row r="71" ht="15.75" customHeight="1" s="31">
       <c r="A71" s="13" t="inlineStr">
         <is>
-          <t>origin</t>
+          <t>sportsbet</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>business analyst</t>
+          <t xml:space="preserve">Graduate Data Scientist Risk &amp; Pricing </t>
         </is>
       </c>
       <c r="C71" s="13" t="inlineStr">
@@ -5813,11 +5812,9 @@
       </c>
       <c r="E71" s="13" t="n"/>
       <c r="F71" s="14" t="n">
-        <v>46166</v>
-      </c>
-      <c r="G71" s="14" t="n">
-        <v>46166</v>
-      </c>
+        <v>46264</v>
+      </c>
+      <c r="G71" s="13" t="n"/>
       <c r="H71" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -5833,7 +5830,7 @@
       <c r="P71" s="13" t="n"/>
       <c r="Q71" s="17" t="n"/>
       <c r="R71" s="18">
-        <f>IF(AND(P71&lt;&gt;"",Q71&lt;&gt;""),Q71-P71,"")</f>
+        <f>IF(AND(P75&lt;&gt;"",Q75&lt;&gt;""),Q75-P75,"")</f>
         <v/>
       </c>
       <c r="S71" s="13" t="n"/>
@@ -5844,32 +5841,24 @@
       <c r="X71" s="13" t="n"/>
       <c r="Y71" s="13" t="n"/>
       <c r="Z71" s="13" t="n"/>
-      <c r="AA71" s="13" t="inlineStr">
-        <is>
-          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
-        </is>
-      </c>
-      <c r="AB71" s="13" t="inlineStr">
-        <is>
-          <t>Customer Churn Forecasting Analysis in Telecom Services, Insurance Risk &amp; Claims Analytics Dashboard, Vendor Performance Analytics Dashboard, Credit Fraud Detection Classifier Analysis</t>
-        </is>
-      </c>
+      <c r="AA71" s="13" t="n"/>
+      <c r="AB71" s="13" t="n"/>
       <c r="AC71" s="13" t="n"/>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="31">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>QBE Insurance</t>
+          <t>Spotlight Retail Group (SRG)</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
         <is>
-          <t>data analytics</t>
+          <t xml:space="preserve">CRM &amp; Loyalty Analyst </t>
         </is>
       </c>
       <c r="C72" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Full-time</t>
         </is>
       </c>
       <c r="D72" s="13" t="inlineStr">
@@ -5878,9 +5867,7 @@
         </is>
       </c>
       <c r="E72" s="13" t="n"/>
-      <c r="F72" s="14" t="n">
-        <v>46253</v>
-      </c>
+      <c r="F72" s="13" t="n"/>
       <c r="G72" s="13" t="n"/>
       <c r="H72" s="13" t="inlineStr">
         <is>
@@ -5897,7 +5884,7 @@
       <c r="P72" s="13" t="n"/>
       <c r="Q72" s="17" t="n"/>
       <c r="R72" s="18">
-        <f>IF(AND(P72&lt;&gt;"",Q72&lt;&gt;""),Q72-P72,"")</f>
+        <f>IF(AND(P76&lt;&gt;"",Q76&lt;&gt;""),Q76-P76,"")</f>
         <v/>
       </c>
       <c r="S72" s="13" t="n"/>
@@ -5915,22 +5902,22 @@
     <row r="73" ht="15.75" customHeight="1" s="31">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">queensland government digital </t>
+          <t>streem</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>Data analytics</t>
+          <t>Junior Media Analyst - Remote</t>
         </is>
       </c>
       <c r="C73" s="13" t="inlineStr">
         <is>
-          <t>Graduate School</t>
+          <t>Full-time</t>
         </is>
       </c>
       <c r="D73" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E73" s="13" t="n"/>
@@ -5951,7 +5938,7 @@
       <c r="P73" s="13" t="n"/>
       <c r="Q73" s="17" t="n"/>
       <c r="R73" s="18">
-        <f>IF(AND(P73&lt;&gt;"",Q73&lt;&gt;""),Q73-P73,"")</f>
+        <f>IF(AND(P77&lt;&gt;"",Q77&lt;&gt;""),Q77-P77,"")</f>
         <v/>
       </c>
       <c r="S73" s="13" t="n"/>
@@ -5969,14 +5956,10 @@
     <row r="74" ht="15.75" customHeight="1" s="31">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>shell</t>
-        </is>
-      </c>
-      <c r="B74" s="13" t="inlineStr">
-        <is>
-          <t>business analyst</t>
-        </is>
-      </c>
+          <t>suncorp</t>
+        </is>
+      </c>
+      <c r="B74" s="13" t="n"/>
       <c r="C74" s="13" t="inlineStr">
         <is>
           <t>Graduate Program</t>
@@ -5990,7 +5973,7 @@
       <c r="E74" s="13" t="n"/>
       <c r="F74" s="14" t="inlineStr">
         <is>
-          <t>sep</t>
+          <t>aug</t>
         </is>
       </c>
       <c r="G74" s="13" t="n"/>
@@ -6009,7 +5992,7 @@
       <c r="P74" s="13" t="n"/>
       <c r="Q74" s="17" t="n"/>
       <c r="R74" s="18">
-        <f>IF(AND(P74&lt;&gt;"",Q74&lt;&gt;""),Q74-P74,"")</f>
+        <f>IF(AND(P78&lt;&gt;"",Q78&lt;&gt;""),Q78-P78,"")</f>
         <v/>
       </c>
       <c r="S74" s="13" t="n"/>
@@ -6027,12 +6010,12 @@
     <row r="75" ht="15.75" customHeight="1" s="31">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>sportsbet</t>
+          <t>ventia</t>
         </is>
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Graduate Data Scientist Risk &amp; Pricing </t>
+          <t>data science &amp; analysics graduate</t>
         </is>
       </c>
       <c r="C75" s="13" t="inlineStr">
@@ -6042,12 +6025,12 @@
       </c>
       <c r="D75" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E75" s="13" t="n"/>
       <c r="F75" s="14" t="n">
-        <v>46264</v>
+        <v>46250</v>
       </c>
       <c r="G75" s="13" t="n"/>
       <c r="H75" s="13" t="inlineStr">
@@ -6062,14 +6045,20 @@
       <c r="M75" s="13" t="n"/>
       <c r="N75" s="13" t="n"/>
       <c r="O75" s="13" t="n"/>
-      <c r="P75" s="13" t="n"/>
+      <c r="P75" s="14" t="n">
+        <v>46047</v>
+      </c>
       <c r="Q75" s="17" t="n"/>
       <c r="R75" s="18">
-        <f>IF(AND(P75&lt;&gt;"",Q75&lt;&gt;""),Q75-P75,"")</f>
+        <f>IF(AND(P79&lt;&gt;"",Q79&lt;&gt;""),Q79-P79,"")</f>
         <v/>
       </c>
       <c r="S75" s="13" t="n"/>
-      <c r="T75" s="13" t="n"/>
+      <c r="T75" s="13" t="inlineStr">
+        <is>
+          <t>70-80k</t>
+        </is>
+      </c>
       <c r="U75" s="20" t="n"/>
       <c r="V75" s="13" t="n"/>
       <c r="W75" s="13" t="n"/>
@@ -6083,17 +6072,17 @@
     <row r="76" ht="15.75" customHeight="1" s="31">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>Spotlight Retail Group (SRG)</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">CRM &amp; Loyalty Analyst </t>
+          <t>data science consulting</t>
         </is>
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Full-time</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
@@ -6119,7 +6108,7 @@
       <c r="P76" s="13" t="n"/>
       <c r="Q76" s="17" t="n"/>
       <c r="R76" s="18">
-        <f>IF(AND(P76&lt;&gt;"",Q76&lt;&gt;""),Q76-P76,"")</f>
+        <f>IF(AND(P80&lt;&gt;"",Q80&lt;&gt;""),Q80-P80,"")</f>
         <v/>
       </c>
       <c r="S76" s="13" t="n"/>
@@ -6137,26 +6126,28 @@
     <row r="77" ht="15.75" customHeight="1" s="31">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>streem</t>
+          <t>visagio</t>
         </is>
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>Junior Media Analyst - Remote</t>
+          <t>data &amp; analytics consultant</t>
         </is>
       </c>
       <c r="C77" s="13" t="inlineStr">
         <is>
-          <t>Full-time</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D77" s="13" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E77" s="13" t="n"/>
-      <c r="F77" s="13" t="n"/>
+      <c r="F77" s="14" t="n">
+        <v>46105</v>
+      </c>
       <c r="G77" s="13" t="n"/>
       <c r="H77" s="13" t="inlineStr">
         <is>
@@ -6173,7 +6164,7 @@
       <c r="P77" s="13" t="n"/>
       <c r="Q77" s="17" t="n"/>
       <c r="R77" s="18">
-        <f>IF(AND(P77&lt;&gt;"",Q77&lt;&gt;""),Q77-P77,"")</f>
+        <f>IF(AND(P81&lt;&gt;"",Q81&lt;&gt;""),Q81-P81,"")</f>
         <v/>
       </c>
       <c r="S77" s="13" t="n"/>
@@ -6191,13 +6182,17 @@
     <row r="78" ht="15.75" customHeight="1" s="31">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>suncorp</t>
-        </is>
-      </c>
-      <c r="B78" s="13" t="n"/>
+          <t>Vistar Media</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Analytics Associate </t>
+        </is>
+      </c>
       <c r="C78" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Full-time</t>
         </is>
       </c>
       <c r="D78" s="13" t="inlineStr">
@@ -6206,11 +6201,7 @@
         </is>
       </c>
       <c r="E78" s="13" t="n"/>
-      <c r="F78" s="14" t="inlineStr">
-        <is>
-          <t>aug</t>
-        </is>
-      </c>
+      <c r="F78" s="13" t="n"/>
       <c r="G78" s="13" t="n"/>
       <c r="H78" s="13" t="inlineStr">
         <is>
@@ -6227,7 +6218,7 @@
       <c r="P78" s="13" t="n"/>
       <c r="Q78" s="17" t="n"/>
       <c r="R78" s="18">
-        <f>IF(AND(P78&lt;&gt;"",Q78&lt;&gt;""),Q78-P78,"")</f>
+        <f>IF(AND(P82&lt;&gt;"",Q82&lt;&gt;""),Q82-P82,"")</f>
         <v/>
       </c>
       <c r="S78" s="13" t="n"/>
@@ -6245,12 +6236,12 @@
     <row r="79" ht="15.75" customHeight="1" s="31">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>ventia</t>
+          <t>Westpac</t>
         </is>
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>data science &amp; analysics graduate</t>
+          <t>Technology (Data)</t>
         </is>
       </c>
       <c r="C79" s="13" t="inlineStr">
@@ -6260,12 +6251,12 @@
       </c>
       <c r="D79" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E79" s="13" t="n"/>
       <c r="F79" s="14" t="n">
-        <v>46250</v>
+        <v>46248</v>
       </c>
       <c r="G79" s="13" t="n"/>
       <c r="H79" s="13" t="inlineStr">
@@ -6280,21 +6271,27 @@
       <c r="M79" s="13" t="n"/>
       <c r="N79" s="13" t="n"/>
       <c r="O79" s="13" t="n"/>
-      <c r="P79" s="14" t="n">
-        <v>46047</v>
+      <c r="P79" s="14" t="inlineStr">
+        <is>
+          <t>1 Feb 2027 - 28 Feb 2027</t>
+        </is>
       </c>
       <c r="Q79" s="17" t="n"/>
       <c r="R79" s="18">
-        <f>IF(AND(P79&lt;&gt;"",Q79&lt;&gt;""),Q79-P79,"")</f>
+        <f>IF(AND(P83&lt;&gt;"",Q83&lt;&gt;""),Q83-P83,"")</f>
         <v/>
       </c>
       <c r="S79" s="13" t="n"/>
       <c r="T79" s="13" t="inlineStr">
         <is>
-          <t>70-80k</t>
-        </is>
-      </c>
-      <c r="U79" s="20" t="n"/>
+          <t>80k-90k</t>
+        </is>
+      </c>
+      <c r="U79" s="20" t="inlineStr">
+        <is>
+          <t>1-100</t>
+        </is>
+      </c>
       <c r="V79" s="13" t="n"/>
       <c r="W79" s="13" t="n"/>
       <c r="X79" s="13" t="n"/>
@@ -6307,12 +6304,12 @@
     <row r="80" ht="15.75" customHeight="1" s="31">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>westpac</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
         <is>
-          <t>data science consulting</t>
+          <t>data digital ai</t>
         </is>
       </c>
       <c r="C80" s="13" t="inlineStr">
@@ -6322,11 +6319,13 @@
       </c>
       <c r="D80" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E80" s="13" t="n"/>
-      <c r="F80" s="13" t="n"/>
+      <c r="F80" s="14" t="n">
+        <v>46248</v>
+      </c>
       <c r="G80" s="13" t="n"/>
       <c r="H80" s="13" t="inlineStr">
         <is>
@@ -6340,14 +6339,20 @@
       <c r="M80" s="13" t="n"/>
       <c r="N80" s="13" t="n"/>
       <c r="O80" s="13" t="n"/>
-      <c r="P80" s="13" t="n"/>
+      <c r="P80" s="14" t="n">
+        <v>46068</v>
+      </c>
       <c r="Q80" s="17" t="n"/>
       <c r="R80" s="18">
-        <f>IF(AND(P80&lt;&gt;"",Q80&lt;&gt;""),Q80-P80,"")</f>
+        <f>IF(AND(P84&lt;&gt;"",Q84&lt;&gt;""),Q84-P84,"")</f>
         <v/>
       </c>
       <c r="S80" s="13" t="n"/>
-      <c r="T80" s="13" t="n"/>
+      <c r="T80" s="13" t="inlineStr">
+        <is>
+          <t>80-90k</t>
+        </is>
+      </c>
       <c r="U80" s="20" t="n"/>
       <c r="V80" s="13" t="n"/>
       <c r="W80" s="13" t="n"/>
@@ -6361,17 +6366,17 @@
     <row r="81" ht="15.75" customHeight="1" s="31">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>visagio</t>
+          <t>evolution mining</t>
         </is>
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
-          <t>data &amp; analytics consultant</t>
+          <t>people and culture</t>
         </is>
       </c>
       <c r="C81" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D81" s="13" t="inlineStr">
@@ -6380,27 +6385,40 @@
         </is>
       </c>
       <c r="E81" s="13" t="n"/>
-      <c r="F81" s="14" t="n">
-        <v>46105</v>
-      </c>
-      <c r="G81" s="13" t="n"/>
+      <c r="F81" s="13" t="n"/>
+      <c r="G81" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H81" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I81" s="13" t="n"/>
-      <c r="J81" s="13" t="n"/>
+      <c r="J81" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K81" s="13" t="n"/>
       <c r="L81" s="13" t="n"/>
-      <c r="M81" s="13" t="n"/>
+      <c r="M81" s="13" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
       <c r="N81" s="13" t="n"/>
       <c r="O81" s="13" t="n"/>
-      <c r="P81" s="13" t="n"/>
+      <c r="P81" s="14" t="inlineStr">
+        <is>
+          <t>12/1/2026 - 12/31/2026</t>
+        </is>
+      </c>
       <c r="Q81" s="17" t="n"/>
-      <c r="R81" s="18">
-        <f>IF(AND(P81&lt;&gt;"",Q81&lt;&gt;""),Q81-P81,"")</f>
-        <v/>
+      <c r="R81" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S81" s="13" t="n"/>
       <c r="T81" s="13" t="n"/>
@@ -6417,47 +6435,68 @@
     <row r="82" ht="15.75" customHeight="1" s="31">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>Vistar Media</t>
+          <t>suncorp</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Analytics Associate </t>
+          <t>business analysis non technical</t>
         </is>
       </c>
       <c r="C82" s="13" t="inlineStr">
         <is>
-          <t>Full-time</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D82" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E82" s="13" t="n"/>
       <c r="F82" s="13" t="n"/>
-      <c r="G82" s="13" t="n"/>
+      <c r="G82" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I82" s="13" t="n"/>
-      <c r="J82" s="13" t="n"/>
-      <c r="K82" s="13" t="n"/>
+      <c r="J82" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K82" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="L82" s="13" t="n"/>
-      <c r="M82" s="13" t="n"/>
+      <c r="M82" s="13" t="inlineStr">
+        <is>
+          <t>Finished Assessment</t>
+        </is>
+      </c>
       <c r="N82" s="13" t="n"/>
       <c r="O82" s="13" t="n"/>
-      <c r="P82" s="13" t="n"/>
-      <c r="Q82" s="17" t="n"/>
-      <c r="R82" s="18">
-        <f>IF(AND(P82&lt;&gt;"",Q82&lt;&gt;""),Q82-P82,"")</f>
-        <v/>
+      <c r="P82" s="14" t="n">
+        <v>46350</v>
+      </c>
+      <c r="Q82" s="17" t="n">
+        <v>46430</v>
+      </c>
+      <c r="R82" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S82" s="13" t="n"/>
-      <c r="T82" s="13" t="n"/>
+      <c r="T82" s="13" t="n">
+        <v>37.92</v>
+      </c>
       <c r="U82" s="20" t="n"/>
       <c r="V82" s="13" t="n"/>
       <c r="W82" s="13" t="n"/>
@@ -6471,60 +6510,67 @@
     <row r="83" ht="15.75" customHeight="1" s="31">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>Westpac</t>
+          <t>ARUP</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>Technology (Data)</t>
+          <t>digital advisory</t>
         </is>
       </c>
       <c r="C83" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="E83" s="13" t="n"/>
-      <c r="F83" s="14" t="n">
-        <v>46248</v>
-      </c>
-      <c r="G83" s="13" t="n"/>
+      <c r="F83" s="13" t="n"/>
+      <c r="G83" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H83" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I83" s="13" t="n"/>
-      <c r="J83" s="13" t="n"/>
+      <c r="J83" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K83" s="13" t="n"/>
       <c r="L83" s="13" t="n"/>
-      <c r="M83" s="13" t="n"/>
+      <c r="M83" s="13" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
       <c r="N83" s="13" t="n"/>
       <c r="O83" s="13" t="n"/>
-      <c r="P83" s="14" t="inlineStr">
-        <is>
-          <t>1 Feb 2027 - 28 Feb 2027</t>
-        </is>
+      <c r="P83" s="14" t="n">
+        <v>46349</v>
       </c>
       <c r="Q83" s="17" t="n"/>
-      <c r="R83" s="18">
-        <f>IF(AND(P83&lt;&gt;"",Q83&lt;&gt;""),Q83-P83,"")</f>
-        <v/>
+      <c r="R83" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S83" s="13" t="n"/>
       <c r="T83" s="13" t="inlineStr">
         <is>
-          <t>80k-90k</t>
+          <t>34-35</t>
         </is>
       </c>
       <c r="U83" s="20" t="inlineStr">
         <is>
-          <t>1-100</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V83" s="13" t="n"/>
@@ -6539,29 +6585,29 @@
     <row r="84" ht="15.75" customHeight="1" s="31">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>westpac</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
         <is>
-          <t>data digital ai</t>
+          <t>data &amp; AI Governance</t>
         </is>
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E84" s="13" t="n"/>
-      <c r="F84" s="14" t="n">
-        <v>46248</v>
-      </c>
-      <c r="G84" s="13" t="n"/>
+      <c r="F84" s="13" t="n"/>
+      <c r="G84" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H84" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -6571,23 +6617,24 @@
       <c r="J84" s="13" t="n"/>
       <c r="K84" s="13" t="n"/>
       <c r="L84" s="13" t="n"/>
-      <c r="M84" s="13" t="n"/>
+      <c r="M84" s="13" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
       <c r="N84" s="13" t="n"/>
       <c r="O84" s="13" t="n"/>
-      <c r="P84" s="14" t="n">
-        <v>46068</v>
+      <c r="P84" s="24" t="n">
+        <v>46356</v>
       </c>
       <c r="Q84" s="17" t="n"/>
-      <c r="R84" s="18">
-        <f>IF(AND(P84&lt;&gt;"",Q84&lt;&gt;""),Q84-P84,"")</f>
-        <v/>
+      <c r="R84" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S84" s="13" t="n"/>
-      <c r="T84" s="13" t="inlineStr">
-        <is>
-          <t>80-90k</t>
-        </is>
-      </c>
+      <c r="T84" s="13" t="n"/>
       <c r="U84" s="20" t="n"/>
       <c r="V84" s="13" t="n"/>
       <c r="W84" s="13" t="n"/>
@@ -6601,49 +6648,71 @@
     <row r="85" ht="15.75" customHeight="1" s="31">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>woolworths group</t>
+          <t>Rheinmetall</t>
         </is>
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
-          <t>graduate product</t>
+          <t>data analytics</t>
         </is>
       </c>
       <c r="C85" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D85" s="13" t="n"/>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D85" s="13" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
       <c r="E85" s="13" t="n"/>
-      <c r="F85" s="14" t="inlineStr">
-        <is>
-          <t>sep</t>
-        </is>
-      </c>
-      <c r="G85" s="13" t="n"/>
+      <c r="F85" s="13" t="n"/>
+      <c r="G85" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H85" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I85" s="13" t="n"/>
-      <c r="J85" s="13" t="n"/>
+      <c r="J85" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K85" s="13" t="n"/>
       <c r="L85" s="13" t="n"/>
       <c r="M85" s="13" t="inlineStr">
         <is>
-          <t>To Apply</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="N85" s="13" t="n"/>
       <c r="O85" s="13" t="n"/>
-      <c r="P85" s="13" t="n"/>
-      <c r="Q85" s="17" t="n"/>
-      <c r="R85" s="28" t="n"/>
+      <c r="P85" s="24" t="n">
+        <v>46349</v>
+      </c>
+      <c r="Q85" s="17" t="n">
+        <v>46437</v>
+      </c>
+      <c r="R85" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
+      </c>
       <c r="S85" s="13" t="n"/>
-      <c r="T85" s="13" t="n"/>
-      <c r="U85" s="20" t="n"/>
+      <c r="T85" s="13" t="inlineStr">
+        <is>
+          <t>36 or 66000</t>
+        </is>
+      </c>
+      <c r="U85" s="20" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
       <c r="V85" s="13" t="n"/>
       <c r="W85" s="13" t="n"/>
       <c r="X85" s="13" t="n"/>
@@ -6656,12 +6725,12 @@
     <row r="86">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>evolution mining</t>
+          <t>grant thornton</t>
         </is>
       </c>
       <c r="B86" s="13" t="inlineStr">
         <is>
-          <t>people and culture</t>
+          <t>business consulting</t>
         </is>
       </c>
       <c r="C86" s="13" t="inlineStr">
@@ -6671,7 +6740,7 @@
       </c>
       <c r="D86" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E86" s="13" t="n"/>
@@ -6685,11 +6754,7 @@
         </is>
       </c>
       <c r="I86" s="13" t="n"/>
-      <c r="J86" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J86" s="13" t="n"/>
       <c r="K86" s="13" t="n"/>
       <c r="L86" s="13" t="n"/>
       <c r="M86" s="13" t="inlineStr">
@@ -6699,20 +6764,26 @@
       </c>
       <c r="N86" s="13" t="n"/>
       <c r="O86" s="13" t="n"/>
-      <c r="P86" s="14" t="inlineStr">
-        <is>
-          <t>12/1/2026 - 12/31/2026</t>
+      <c r="P86" s="27" t="inlineStr">
+        <is>
+          <t>11/16/2026 - 18 jan 2027</t>
         </is>
       </c>
       <c r="Q86" s="17" t="n"/>
       <c r="R86" s="28" t="inlineStr">
         <is>
-          <t>12 weeks</t>
+          <t>4-6 weeks</t>
         </is>
       </c>
       <c r="S86" s="13" t="n"/>
-      <c r="T86" s="13" t="n"/>
-      <c r="U86" s="20" t="n"/>
+      <c r="T86" s="13" t="n">
+        <v>278</v>
+      </c>
+      <c r="U86" s="20" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
       <c r="V86" s="13" t="n"/>
       <c r="W86" s="13" t="n"/>
       <c r="X86" s="13" t="n"/>
@@ -6725,12 +6796,12 @@
     <row r="87">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>suncorp</t>
+          <t>nab</t>
         </is>
       </c>
       <c r="B87" s="13" t="inlineStr">
         <is>
-          <t>business analysis non technical</t>
+          <t>digital data and ai</t>
         </is>
       </c>
       <c r="C87" s="13" t="inlineStr">
@@ -6740,7 +6811,7 @@
       </c>
       <c r="D87" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E87" s="13" t="n"/>
@@ -6754,40 +6825,36 @@
         </is>
       </c>
       <c r="I87" s="13" t="n"/>
-      <c r="J87" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K87" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="J87" s="13" t="n"/>
+      <c r="K87" s="13" t="n"/>
       <c r="L87" s="13" t="n"/>
       <c r="M87" s="13" t="inlineStr">
         <is>
-          <t>Finished Assessment</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="N87" s="13" t="n"/>
       <c r="O87" s="13" t="n"/>
-      <c r="P87" s="14" t="n">
-        <v>46350</v>
-      </c>
-      <c r="Q87" s="17" t="n">
-        <v>46430</v>
-      </c>
+      <c r="P87" s="24" t="n">
+        <v>46349</v>
+      </c>
+      <c r="Q87" s="17" t="n"/>
       <c r="R87" s="28" t="inlineStr">
         <is>
-          <t>12 weeks</t>
+          <t>8 weeks</t>
         </is>
       </c>
       <c r="S87" s="13" t="n"/>
-      <c r="T87" s="13" t="n">
-        <v>37.92</v>
-      </c>
-      <c r="U87" s="20" t="n"/>
+      <c r="T87" s="13" t="inlineStr">
+        <is>
+          <t>65000-70000</t>
+        </is>
+      </c>
+      <c r="U87" s="20" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
       <c r="V87" s="13" t="n"/>
       <c r="W87" s="13" t="n"/>
       <c r="X87" s="13" t="n"/>
@@ -6800,12 +6867,12 @@
     <row r="88">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>ARUP</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>digital advisory</t>
+          <t>project management</t>
         </is>
       </c>
       <c r="C88" s="13" t="inlineStr">
@@ -6815,7 +6882,7 @@
       </c>
       <c r="D88" s="13" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E88" s="13" t="n"/>
@@ -6829,11 +6896,7 @@
         </is>
       </c>
       <c r="I88" s="13" t="n"/>
-      <c r="J88" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="J88" s="13" t="n"/>
       <c r="K88" s="13" t="n"/>
       <c r="L88" s="13" t="n"/>
       <c r="M88" s="13" t="inlineStr">
@@ -6843,8 +6906,8 @@
       </c>
       <c r="N88" s="13" t="n"/>
       <c r="O88" s="13" t="n"/>
-      <c r="P88" s="14" t="n">
-        <v>46349</v>
+      <c r="P88" s="24" t="n">
+        <v>46342</v>
       </c>
       <c r="Q88" s="17" t="n"/>
       <c r="R88" s="28" t="inlineStr">
@@ -6853,14 +6916,12 @@
         </is>
       </c>
       <c r="S88" s="13" t="n"/>
-      <c r="T88" s="13" t="inlineStr">
-        <is>
-          <t>34-35</t>
-        </is>
+      <c r="T88" s="13" t="n">
+        <v>38</v>
       </c>
       <c r="U88" s="20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="V88" s="13" t="n"/>
@@ -6875,12 +6936,12 @@
     <row r="89">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>Commonwealth Bank</t>
         </is>
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>data &amp; AI Governance</t>
+          <t>Technology &amp; AI -advanced Analytics</t>
         </is>
       </c>
       <c r="C89" s="13" t="inlineStr">
@@ -6890,13 +6951,15 @@
       </c>
       <c r="D89" s="13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E89" s="13" t="n"/>
-      <c r="F89" s="13" t="n"/>
-      <c r="G89" s="14" t="n">
-        <v>46096</v>
+      <c r="F89" s="24" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G89" s="29" t="n">
+        <v>46272</v>
       </c>
       <c r="H89" s="13" t="inlineStr">
         <is>
@@ -6915,17 +6978,23 @@
       <c r="N89" s="13" t="n"/>
       <c r="O89" s="13" t="n"/>
       <c r="P89" s="24" t="n">
-        <v>46356</v>
-      </c>
-      <c r="Q89" s="17" t="n"/>
+        <v>46349</v>
+      </c>
+      <c r="Q89" s="13" t="n"/>
       <c r="R89" s="28" t="inlineStr">
         <is>
-          <t>12 weeks</t>
+          <t>10 weeks</t>
         </is>
       </c>
       <c r="S89" s="13" t="n"/>
-      <c r="T89" s="13" t="n"/>
-      <c r="U89" s="20" t="n"/>
+      <c r="T89" s="26" t="n">
+        <v>65000</v>
+      </c>
+      <c r="U89" s="20" t="inlineStr">
+        <is>
+          <t>1-8</t>
+        </is>
+      </c>
       <c r="V89" s="13" t="n"/>
       <c r="W89" s="13" t="n"/>
       <c r="X89" s="13" t="n"/>
@@ -6936,431 +7005,255 @@
       <c r="AC89" s="13" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="13" t="inlineStr">
-        <is>
-          <t>Rheinmetall</t>
-        </is>
-      </c>
-      <c r="B90" s="13" t="inlineStr">
-        <is>
-          <t>data analytics</t>
-        </is>
-      </c>
-      <c r="C90" s="13" t="inlineStr">
+      <c r="A90" s="32" t="inlineStr">
+        <is>
+          <t>australian secruity intelligence organisation asio</t>
+        </is>
+      </c>
+      <c r="B90" s="32" t="inlineStr">
+        <is>
+          <t>intelligence development program itelligence analyst</t>
+        </is>
+      </c>
+      <c r="C90" s="32" t="inlineStr">
+        <is>
+          <t>Graduate Program</t>
+        </is>
+      </c>
+      <c r="D90" s="32" t="inlineStr">
+        <is>
+          <t>ACT</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="n">
+        <v>46258</v>
+      </c>
+      <c r="G90" s="6" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H90" s="13" t="inlineStr">
+        <is>
+          <t>Prosple</t>
+        </is>
+      </c>
+      <c r="M90" s="32" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="P90" s="6" t="inlineStr">
+        <is>
+          <t>ongoing</t>
+        </is>
+      </c>
+      <c r="T90" s="32" t="inlineStr">
+        <is>
+          <t>100425 - 125060</t>
+        </is>
+      </c>
+      <c r="U90" s="7" t="inlineStr">
+        <is>
+          <t>5-50</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="32" t="inlineStr">
+        <is>
+          <t>accenture</t>
+        </is>
+      </c>
+      <c r="B91" s="32" t="inlineStr">
+        <is>
+          <t>graduate analyst technology</t>
+        </is>
+      </c>
+      <c r="C91" s="32" t="inlineStr">
+        <is>
+          <t>Graduate Program</t>
+        </is>
+      </c>
+      <c r="D91" s="32" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>46264</v>
+      </c>
+      <c r="H91" s="32" t="inlineStr">
+        <is>
+          <t>Prosple</t>
+        </is>
+      </c>
+      <c r="M91" s="32" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="P91" s="6" t="inlineStr">
+        <is>
+          <t>1/19/2027 - 7/13/2027</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>70000-80000</t>
+        </is>
+      </c>
+      <c r="U91" s="7" t="inlineStr">
+        <is>
+          <t>1-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="32" t="inlineStr">
+        <is>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>business data analyst project intern (GBS)</t>
+        </is>
+      </c>
+      <c r="C92" s="32" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="D90" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E90" s="13" t="n"/>
-      <c r="F90" s="13" t="n"/>
-      <c r="G90" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H90" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I90" s="13" t="n"/>
-      <c r="J90" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K90" s="13" t="n"/>
-      <c r="L90" s="13" t="n"/>
-      <c r="M90" s="13" t="inlineStr">
+      <c r="D92" s="32" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="n">
+        <v>46387</v>
+      </c>
+      <c r="G92" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H92" s="13" t="inlineStr">
+        <is>
+          <t>Prosple</t>
+        </is>
+      </c>
+      <c r="M92" s="32" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="N90" s="13" t="n"/>
-      <c r="O90" s="13" t="n"/>
-      <c r="P90" s="24" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q90" s="17" t="n">
-        <v>46437</v>
-      </c>
-      <c r="R90" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S90" s="13" t="n"/>
-      <c r="T90" s="13" t="inlineStr">
-        <is>
-          <t>36 or 66000</t>
-        </is>
-      </c>
-      <c r="U90" s="20" t="inlineStr">
-        <is>
-          <t>5-6</t>
-        </is>
-      </c>
-      <c r="V90" s="13" t="n"/>
-      <c r="W90" s="13" t="n"/>
-      <c r="X90" s="13" t="n"/>
-      <c r="Y90" s="13" t="n"/>
-      <c r="Z90" s="13" t="n"/>
-      <c r="AA90" s="13" t="n"/>
-      <c r="AB90" s="13" t="n"/>
-      <c r="AC90" s="13" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="13" t="inlineStr">
-        <is>
-          <t>grant thornton</t>
-        </is>
-      </c>
-      <c r="B91" s="13" t="inlineStr">
-        <is>
-          <t>business consulting</t>
-        </is>
-      </c>
-      <c r="C91" s="13" t="inlineStr">
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>2000-5000 per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="32" t="inlineStr">
+        <is>
+          <t>Didi</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="inlineStr">
+        <is>
+          <t>operations intern</t>
+        </is>
+      </c>
+      <c r="C93" s="32" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="D91" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E91" s="13" t="n"/>
-      <c r="F91" s="13" t="n"/>
-      <c r="G91" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H91" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I91" s="13" t="n"/>
-      <c r="J91" s="13" t="n"/>
-      <c r="K91" s="13" t="n"/>
-      <c r="L91" s="13" t="n"/>
-      <c r="M91" s="13" t="inlineStr">
+      <c r="D93" s="32" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="G93" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="M93" s="32" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="N91" s="13" t="n"/>
-      <c r="O91" s="13" t="n"/>
-      <c r="P91" s="27" t="inlineStr">
-        <is>
-          <t>11/16/2026 - 18 jan 2027</t>
-        </is>
-      </c>
-      <c r="Q91" s="17" t="n"/>
-      <c r="R91" s="28" t="inlineStr">
-        <is>
-          <t>4-6 weeks</t>
-        </is>
-      </c>
-      <c r="S91" s="13" t="n"/>
-      <c r="T91" s="13" t="n">
-        <v>278</v>
-      </c>
-      <c r="U91" s="20" t="inlineStr">
-        <is>
-          <t>1-10</t>
-        </is>
-      </c>
-      <c r="V91" s="13" t="n"/>
-      <c r="W91" s="13" t="n"/>
-      <c r="X91" s="13" t="n"/>
-      <c r="Y91" s="13" t="n"/>
-      <c r="Z91" s="13" t="n"/>
-      <c r="AA91" s="13" t="n"/>
-      <c r="AB91" s="13" t="n"/>
-      <c r="AC91" s="13" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="13" t="inlineStr">
-        <is>
-          <t>nab</t>
-        </is>
-      </c>
-      <c r="B92" s="13" t="inlineStr">
-        <is>
-          <t>digital data and ai</t>
-        </is>
-      </c>
-      <c r="C92" s="13" t="inlineStr">
+    </row>
+    <row r="94">
+      <c r="A94" s="32" t="inlineStr">
+        <is>
+          <t>tencent</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Game Reaserch Development intern, engine reasearch</t>
+        </is>
+      </c>
+      <c r="C94" s="32" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="D92" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E92" s="13" t="n"/>
-      <c r="F92" s="13" t="n"/>
-      <c r="G92" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H92" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I92" s="13" t="n"/>
-      <c r="J92" s="13" t="n"/>
-      <c r="K92" s="13" t="n"/>
-      <c r="L92" s="13" t="n"/>
-      <c r="M92" s="13" t="inlineStr">
-        <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="N92" s="13" t="n"/>
-      <c r="O92" s="13" t="n"/>
-      <c r="P92" s="24" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q92" s="17" t="n"/>
-      <c r="R92" s="28" t="inlineStr">
-        <is>
-          <t>8 weeks</t>
-        </is>
-      </c>
-      <c r="S92" s="13" t="n"/>
-      <c r="T92" s="13" t="inlineStr">
-        <is>
-          <t>65000-70000</t>
-        </is>
-      </c>
-      <c r="U92" s="20" t="inlineStr">
-        <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="V92" s="13" t="n"/>
-      <c r="W92" s="13" t="n"/>
-      <c r="X92" s="13" t="n"/>
-      <c r="Y92" s="13" t="n"/>
-      <c r="Z92" s="13" t="n"/>
-      <c r="AA92" s="13" t="n"/>
-      <c r="AB92" s="13" t="n"/>
-      <c r="AC92" s="13" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="13" t="inlineStr">
-        <is>
-          <t>AECOM</t>
-        </is>
-      </c>
-      <c r="B93" s="13" t="inlineStr">
-        <is>
-          <t>project management</t>
-        </is>
-      </c>
-      <c r="C93" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D93" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E93" s="13" t="n"/>
-      <c r="F93" s="13" t="n"/>
-      <c r="G93" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H93" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I93" s="13" t="n"/>
-      <c r="J93" s="13" t="n"/>
-      <c r="K93" s="13" t="n"/>
-      <c r="L93" s="13" t="n"/>
-      <c r="M93" s="13" t="inlineStr">
+      <c r="D94" s="32" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="G94" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="M94" s="32" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="N93" s="13" t="n"/>
-      <c r="O93" s="13" t="n"/>
-      <c r="P93" s="24" t="n">
-        <v>46342</v>
-      </c>
-      <c r="Q93" s="17" t="n"/>
-      <c r="R93" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S93" s="13" t="n"/>
-      <c r="T93" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="U93" s="20" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
-      <c r="V93" s="13" t="n"/>
-      <c r="W93" s="13" t="n"/>
-      <c r="X93" s="13" t="n"/>
-      <c r="Y93" s="13" t="n"/>
-      <c r="Z93" s="13" t="n"/>
-      <c r="AA93" s="13" t="n"/>
-      <c r="AB93" s="13" t="n"/>
-      <c r="AC93" s="13" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="13" t="inlineStr">
-        <is>
-          <t>Commonwealth Bank</t>
-        </is>
-      </c>
-      <c r="B94" s="13" t="inlineStr">
-        <is>
-          <t>Technology &amp; AI -advanced Analytics</t>
-        </is>
-      </c>
-      <c r="C94" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D94" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E94" s="13" t="n"/>
-      <c r="F94" s="24" t="n">
-        <v>46273</v>
-      </c>
-      <c r="G94" s="29" t="n">
-        <v>46272</v>
-      </c>
-      <c r="H94" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I94" s="13" t="n"/>
-      <c r="J94" s="13" t="n"/>
-      <c r="K94" s="13" t="n"/>
-      <c r="L94" s="13" t="n"/>
-      <c r="M94" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N94" s="13" t="n"/>
-      <c r="O94" s="13" t="n"/>
-      <c r="P94" s="24" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q94" s="13" t="n"/>
-      <c r="R94" s="28" t="inlineStr">
-        <is>
-          <t>10 weeks</t>
-        </is>
-      </c>
-      <c r="S94" s="13" t="n"/>
-      <c r="T94" s="26" t="n">
-        <v>65000</v>
-      </c>
-      <c r="U94" s="20" t="inlineStr">
-        <is>
-          <t>1-8</t>
-        </is>
-      </c>
-      <c r="V94" s="13" t="n"/>
-      <c r="W94" s="13" t="n"/>
-      <c r="X94" s="13" t="n"/>
-      <c r="Y94" s="13" t="n"/>
-      <c r="Z94" s="13" t="n"/>
-      <c r="AA94" s="13" t="n"/>
-      <c r="AB94" s="13" t="n"/>
-      <c r="AC94" s="13" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="32" t="inlineStr">
         <is>
-          <t>australian secruity intelligence organisation asio</t>
-        </is>
-      </c>
-      <c r="B95" s="32" t="inlineStr">
-        <is>
-          <t>intelligence development program itelligence analyst</t>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>information systems and technology</t>
         </is>
       </c>
       <c r="C95" s="32" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D95" s="32" t="inlineStr">
         <is>
-          <t>ACT</t>
-        </is>
-      </c>
-      <c r="F95" s="6" t="n">
-        <v>46258</v>
-      </c>
-      <c r="G95" s="6" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H95" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="G95" s="34" t="n">
+        <v>46277</v>
       </c>
       <c r="M95" s="32" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="P95" s="6" t="inlineStr">
-        <is>
-          <t>ongoing</t>
-        </is>
-      </c>
-      <c r="T95" s="32" t="inlineStr">
-        <is>
-          <t>100425 - 125060</t>
-        </is>
-      </c>
-      <c r="U95" s="7" t="inlineStr">
-        <is>
-          <t>5-50</t>
+          <t>Applied</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="32" t="inlineStr">
         <is>
-          <t>accenture</t>
-        </is>
-      </c>
-      <c r="B96" s="32" t="inlineStr">
-        <is>
-          <t>graduate analyst technology</t>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>student training and totation program intern</t>
         </is>
       </c>
       <c r="C96" s="32" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D96" s="32" t="inlineStr">
@@ -7368,373 +7261,17 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="F96" s="6" t="n">
-        <v>46264</v>
-      </c>
-      <c r="H96" s="32" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
+      <c r="G96" s="34" t="n">
+        <v>46277</v>
       </c>
       <c r="M96" s="32" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="P96" s="6" t="inlineStr">
-        <is>
-          <t>1/19/2027 - 7/13/2027</t>
-        </is>
-      </c>
-      <c r="T96" t="inlineStr">
-        <is>
-          <t>70000-80000</t>
-        </is>
-      </c>
-      <c r="U96" s="7" t="inlineStr">
-        <is>
-          <t>1-45</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">queensland government digital </t>
-        </is>
-      </c>
-      <c r="C97" s="32" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D97" s="32" t="inlineStr">
-        <is>
-          <t>QLD</t>
-        </is>
-      </c>
-      <c r="E97" s="6" t="n">
-        <v>46265</v>
-      </c>
-      <c r="F97" s="6" t="n">
-        <v>46278</v>
-      </c>
-      <c r="H97" s="32" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="M97" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-      <c r="P97" s="6" t="n">
-        <v>46419</v>
-      </c>
-      <c r="T97" t="inlineStr">
-        <is>
-          <t>76216-84571</t>
-        </is>
-      </c>
-      <c r="U97" s="7" t="inlineStr">
-        <is>
-          <t>30-80</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="32" t="inlineStr">
-        <is>
-          <t>loreal</t>
-        </is>
-      </c>
-      <c r="C98" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D98" s="32" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E98" s="6" t="n">
-        <v>46266</v>
-      </c>
-      <c r="F98" s="6" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H98" s="32" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="M98" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-      <c r="P98" s="6" t="n">
-        <v>46398</v>
-      </c>
-      <c r="R98" t="inlineStr">
-        <is>
-          <t>6 months</t>
-        </is>
-      </c>
-      <c r="T98" t="inlineStr">
-        <is>
-          <t>45000 - 50000</t>
-        </is>
-      </c>
-      <c r="U98" s="7" t="inlineStr">
-        <is>
-          <t>1-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="32" t="inlineStr">
-        <is>
-          <t>tiktok</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>business data analyst project intern (GBS)</t>
-        </is>
-      </c>
-      <c r="C99" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D99" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="F99" s="6" t="n">
-        <v>46387</v>
-      </c>
-      <c r="H99" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="M99" s="32" t="inlineStr">
-        <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="T99" t="inlineStr">
-        <is>
-          <t>2000-5000 per month</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="32" t="inlineStr">
-        <is>
-          <t>Futures Sport &amp; entertainment</t>
-        </is>
-      </c>
-      <c r="B100" s="32" t="inlineStr">
-        <is>
-          <t>Sports Consultancy and data analyst intern</t>
-        </is>
-      </c>
-      <c r="C100" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D100" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="H100" s="32" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="M100" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="32" t="inlineStr">
-        <is>
-          <t>Didi</t>
-        </is>
-      </c>
-      <c r="B101" s="32" t="inlineStr">
-        <is>
-          <t>operations intern</t>
-        </is>
-      </c>
-      <c r="C101" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D101" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="M101" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="32" t="inlineStr">
-        <is>
-          <t>tencent</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Game Reaserch Development intern, engine reasearch</t>
-        </is>
-      </c>
-      <c r="C102" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D102" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="M102" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="32" t="inlineStr">
-        <is>
-          <t>apple</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>information systems and technology</t>
-        </is>
-      </c>
-      <c r="C103" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D103" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="M103" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="32" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>student training and totation program intern</t>
-        </is>
-      </c>
-      <c r="C104" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D104" s="32" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="M104" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-      <c r="R104" t="inlineStr">
+      <c r="R96" t="inlineStr">
         <is>
           <t>2 years</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="32" t="inlineStr">
-        <is>
-          <t>bytedance</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>ai sales intern</t>
-        </is>
-      </c>
-      <c r="C105" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D105" s="32" t="inlineStr">
-        <is>
-          <t>Hong Kong</t>
-        </is>
-      </c>
-      <c r="M105" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="32" t="inlineStr">
-        <is>
-          <t>binance</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>BAP data analyst</t>
-        </is>
-      </c>
-      <c r="C106" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D106" s="32" t="inlineStr">
-        <is>
-          <t>Hong Kong</t>
-        </is>
-      </c>
-      <c r="M106" s="32" t="inlineStr">
-        <is>
-          <t>To Apply</t>
-        </is>
-      </c>
-      <c r="R106" t="inlineStr">
-        <is>
-          <t>3 month</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
job-tracker: remove leftover Acme Analytics template answers
Two Answers-sheet rows for "Acme Analytics / Graduate Data Analyst" had
no matching Applications row and were never a real application —
leftover template content from setting up the tracker. Confirmed with
Eileen and removed; generate_job_data.py no longer warns about them.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -7541,7 +7541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="31" min="1" max="1"/>
@@ -7579,58 +7579,18 @@
       </c>
     </row>
     <row r="2" ht="60" customHeight="1" s="31">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Acme Analytics</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Graduate Data Analyst</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Why have you chosen to apply to Acme Analytics?</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>mission, growth</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Acme's focus on using data to improve public transit access lines up with why I got into analytics in the first place - I want my work to have a visible, everyday impact.</t>
-        </is>
-      </c>
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="n"/>
     </row>
     <row r="3" ht="60" customHeight="1" s="31">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Acme Analytics</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Graduate Data Analyst</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>How &lt;company&gt; aligns with your personal aspirations?</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>mission, culture, mentorship</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>I'm looking for a graduate program with structured mentorship and rotational exposure across teams, which is exactly how Acme's program is set up.</t>
-        </is>
-      </c>
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n"/>
@@ -7870,20 +7830,6 @@
       <c r="D37" s="5" t="n"/>
       <c r="E37" s="5" t="n"/>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="n"/>
-      <c r="B38" s="5" t="n"/>
-      <c r="C38" s="5" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="5" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="n"/>
-      <c r="B39" s="5" t="n"/>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:E40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>